<commit_message>
[Merging] data dictionary — technical and identifier columns
Fills meaning + notes for all 65 CONSTANT / UNIQUE_ID / ALL_MISSING rows
across six study sheets. Covers SRA/ENA archive boilerplate (run/experiment/
BioSample/BioProject accessions, platform, library layout, organism, etc.)
and clinically constant cohort fields (sirolimus, myeloabl, cgvhd, thiotepa
dose, graft manipulation, bosutinib indicators). PATIENT_LEVEL and
SAMPLE_LEVEL rows are untouched. Cohort-homogeneous CONSTANT columns flagged
UNCERTAIN in notes where relevant. Script: Merging/fill_technical_meanings.R.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Merging/data_dictionaries.xlsx
+++ b/Merging/data_dictionaries.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="453">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="546">
   <si>
     <t xml:space="preserve">column_name</t>
   </si>
@@ -1376,6 +1376,285 @@
   </si>
   <si>
     <t xml:space="preserve">pos/pos | neg/neg | neg/pos | pos/neg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QIIME2 primary sample identifier; equals the SRA run accession (SRR) for this study</t>
+  </si>
+  <si>
+    <t xml:space="preserve">unique per sample — identifier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRA run accession (SRR...); unique per sequencing run, identical to sample-id here</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRA experiment accession (SRX...); groups runs from the same library preparation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRA submitter-assigned library name; encodes patient ID and timepoint (e.g., 59_post_16S)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRA library assay-type classification; value 'WGA' (whole-genome amplification) is SRA's generic label for amplicon libraries submitted without an explicit amplicon assay type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: WGA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total number of bases sequenced in the SRA run (bp)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NCBI BioProject accession for this study (PRJNA592853)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: PRJNA592853</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NCBI BioSample accession (SAMN...); unique per physical sample in NCBI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NCBI BioSample metadata schema applied to these submissions; 'Metagenome or environmental' is the standard schema for gut microbiome samples</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: Metagenome or environmental</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compressed file size of the SRA run data (bytes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name of the institution that submitted the data to SRA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: UNIVERSITY OF BOLOGNA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sample collection date as recorded in SRA metadata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: not available — date not provided by submitters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRA data-access consent classification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: public</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRA experiment accession (SRX...); unique per sequencing library</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Country of sample collection as recorded in SRA metadata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: Italy — UNCERTAIN: constant in this study but analytically meaningful — may vary across studies at merge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Continent of sample collection as recorded in SRA metadata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: Europe — UNCERTAIN: constant in this study but analytically meaningful — may vary across studies at merge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Geographic location (country:city) of sample collection as recorded in SRA metadata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: Italy:Bologna — UNCERTAIN: constant in this study but analytically meaningful — may vary across studies at merge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Host organism for the microbiome sample as recorded in NCBI taxonomy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: Homo sapiens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Submitter-assigned host (patient) identifier in SRA; equivalent to patient ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sequencing instrument model used for this study</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: Illumina MiSeq</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sample source material as recorded in SRA metadata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: human feces</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biological source from which the sample was isolated, as recorded in SRA metadata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: human gut</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latitude/longitude of sample collection site as recorded in SRA metadata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: missing — coordinates not provided by submitters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Submitter-assigned library name in SRA; corresponds to the patient identifier used in the study</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sequencing read layout: single-end or paired-end</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: SINGLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Method used to select or enrich the sequencing library (PCR = PCR amplification, as expected for 16S amplicon libraries)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: PCR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Type of source material sequenced as recorded in SRA; GENOMIC is SRA's label for amplicon libraries lacking an explicit AMPLICON source type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: GENOMIC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NCBI taxonomy label applied to the sample</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: human gut metagenome</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sequencing technology platform</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: ILLUMINA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRA metadata schema version number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Submitter-defined sample name in SRA; identical to Library Name and HostID for this study</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sample type classification as recorded in SRA metadata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: metagenomic assembly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRA study accession; groups all runs from the same BioProject submission (SRP234378)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: SRP234378</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Descriptive sample name encoding patient ID and timepoint (e.g., OCUBMT001_day0); submitter-defined</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Duplicate of sample-id; SRA run accession (SRR...) assigned by submitters as a redundant identifier column</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QIIME2 primary sample identifier; equals the ENA run accession (ERR) for this study</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENA run accession (ERR...); unique per sequencing run, identical to sample-id here</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENA run accession (ERR...); duplicate of Run and sample-id columns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENA sample accession (SAMEA...); unique per physical sample in ENA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENA experiment accession (ERX...); groups runs from the same library preparation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENA secondary sample accession (ERS...); alternative stable identifier for the sample in the European Nucleotide Archive</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENA external sample identifier; identical to sample_accession (SAMEA...) for this study</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generic library name assigned by the submitter (Sample1, Sample2, …); no study-specific information encoded</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Descriptive ENA sample title encoding patient ID and visit/week (e.g., P01.w1); submitter-defined</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Day of GvHD onset relative to transplant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">all values missing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Binary indicator: was the graft manipulated (e.g., T-cell depletion) for GvHD prophylaxis (0 = no)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: 0 — UNCERTAIN: constant in this study but analytically meaningful — may vary across studies at merge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Binary indicator: did the patient develop chronic GvHD (0 = no)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Study-internal flag; exact meaning unknown; value 'no' for all samples</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: no — UNCERTAIN: constant in this study but analytically meaningful — may vary across studies at merge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Binary indicator: did the patient receive myeloablative conditioning (1 = yes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: 1 — UNCERTAIN: constant in this study but analytically meaningful — may vary across studies at merge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total dose of thiotepa (mg) given as part of the conditioning regimen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QIIME2 primary sample identifier; equals the ENA BioSample accession (SAMEA) for this study</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENA BioSample accession (SAMEA...); identical to sample-id and sample_accession for this study</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Submitter-assigned library name in ENA/SRA; encodes study ID and patient ID (e.g., 10564.0QP6NJCM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENA sample accession (SAMEA...); identical to sample-id and BioSample for this study</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient identifier used as the patient key for this study</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENA external sample identifier; identical to BioSample and sample_accession (SAMEA...) for this study</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Binary indicator: did the patient receive sirolimus as GvHD prophylaxis (no = none received)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Study-specific sample identifier used as the patient key; encodes patient code, sample date, and a suffix (e.g., 002-1101-G-D_12_05_14)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Administrative field: whether the patient withdrew study consent (no = consent retained)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: no — administrative field, not analytically meaningful</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Study-internal field; exact meaning unknown; possibly a version or protocol code related to bosutinib arm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: 2,62 — UNCERTAIN: constant in this study but analytically meaningful — may vary across studies at merge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date associated with bosutinib treatment or protocol event (format YYYY-MM-DD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: 2016-03-07 — UNCERTAIN: constant in this study but analytically meaningful — may vary across studies at merge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Binary indicator: patient enrolled in or received bosutinib (yes = all patients in this exported subset received bosutinib)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constant across all samples; constant value: yes — UNCERTAIN: constant in this study but analytically meaningful — may vary across studies at merge</t>
   </si>
 </sst>
 </file>
@@ -1804,10 +2083,14 @@
       <c r="G2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="2"/>
+      <c r="H2" s="2" t="s">
+        <v>453</v>
+      </c>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
+      <c r="K2" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="2" t="s">
@@ -1831,10 +2114,14 @@
       <c r="G3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="2"/>
+      <c r="H3" s="2" t="s">
+        <v>455</v>
+      </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
+      <c r="K3" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="s">
@@ -1858,10 +2145,14 @@
       <c r="G4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="H4" s="2"/>
+      <c r="H4" s="2" t="s">
+        <v>456</v>
+      </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
+      <c r="K4" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="2" t="s">
@@ -1885,10 +2176,14 @@
       <c r="G5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H5" s="2"/>
+      <c r="H5" s="2" t="s">
+        <v>457</v>
+      </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
+      <c r="K5" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="2" t="s">
@@ -2565,10 +2860,14 @@
       <c r="G2" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="H2" s="2"/>
+      <c r="H2" s="2" t="s">
+        <v>453</v>
+      </c>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
+      <c r="K2" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="2" t="s">
@@ -2592,10 +2891,14 @@
       <c r="G3" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="H3" s="2"/>
+      <c r="H3" s="2" t="s">
+        <v>458</v>
+      </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
+      <c r="K3" s="2" t="s">
+        <v>459</v>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="s">
@@ -2646,10 +2949,14 @@
       <c r="G5" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="H5" s="2"/>
+      <c r="H5" s="2" t="s">
+        <v>460</v>
+      </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
+      <c r="K5" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="2" t="s">
@@ -2673,10 +2980,14 @@
       <c r="G6" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="H6" s="2"/>
+      <c r="H6" s="2" t="s">
+        <v>461</v>
+      </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
+      <c r="K6" s="2" t="s">
+        <v>462</v>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="2" t="s">
@@ -2700,10 +3011,14 @@
       <c r="G7" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="H7" s="2"/>
+      <c r="H7" s="2" t="s">
+        <v>463</v>
+      </c>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
+      <c r="K7" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="2" t="s">
@@ -2727,10 +3042,14 @@
       <c r="G8" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="H8" s="2"/>
+      <c r="H8" s="2" t="s">
+        <v>464</v>
+      </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
+      <c r="K8" s="2" t="s">
+        <v>465</v>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="2" t="s">
@@ -2754,10 +3073,14 @@
       <c r="G9" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="H9" s="2"/>
+      <c r="H9" s="2" t="s">
+        <v>466</v>
+      </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
+      <c r="K9" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="2" t="s">
@@ -2781,10 +3104,14 @@
       <c r="G10" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="H10" s="2"/>
+      <c r="H10" s="2" t="s">
+        <v>467</v>
+      </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
+      <c r="K10" s="2" t="s">
+        <v>468</v>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="2" t="s">
@@ -2808,10 +3135,14 @@
       <c r="G11" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="H11" s="2"/>
+      <c r="H11" s="2" t="s">
+        <v>469</v>
+      </c>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
+      <c r="K11" s="2" t="s">
+        <v>470</v>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="2" t="s">
@@ -2835,10 +3166,14 @@
       <c r="G12" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="H12" s="2"/>
+      <c r="H12" s="2" t="s">
+        <v>471</v>
+      </c>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
-      <c r="K12" s="2"/>
+      <c r="K12" s="2" t="s">
+        <v>472</v>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="2" t="s">
@@ -2943,10 +3278,14 @@
       <c r="G16" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="H16" s="2"/>
+      <c r="H16" s="2" t="s">
+        <v>473</v>
+      </c>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
+      <c r="K16" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="2" t="s">
@@ -2970,10 +3309,14 @@
       <c r="G17" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="H17" s="2"/>
+      <c r="H17" s="2" t="s">
+        <v>474</v>
+      </c>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
+      <c r="K17" s="2" t="s">
+        <v>475</v>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="2" t="s">
@@ -2997,10 +3340,14 @@
       <c r="G18" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="H18" s="2"/>
+      <c r="H18" s="2" t="s">
+        <v>476</v>
+      </c>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
-      <c r="K18" s="2"/>
+      <c r="K18" s="2" t="s">
+        <v>477</v>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="2" t="s">
@@ -3024,10 +3371,14 @@
       <c r="G19" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="H19" s="2"/>
+      <c r="H19" s="2" t="s">
+        <v>478</v>
+      </c>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
-      <c r="K19" s="2"/>
+      <c r="K19" s="2" t="s">
+        <v>479</v>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="2" t="s">
@@ -3051,10 +3402,14 @@
       <c r="G20" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="H20" s="2"/>
+      <c r="H20" s="2" t="s">
+        <v>480</v>
+      </c>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
-      <c r="K20" s="2"/>
+      <c r="K20" s="2" t="s">
+        <v>481</v>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="2" t="s">
@@ -3078,10 +3433,14 @@
       <c r="G21" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="H21" s="2"/>
+      <c r="H21" s="2" t="s">
+        <v>482</v>
+      </c>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
-      <c r="K21" s="2"/>
+      <c r="K21" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="2" t="s">
@@ -3105,10 +3464,14 @@
       <c r="G22" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="H22" s="2"/>
+      <c r="H22" s="2" t="s">
+        <v>483</v>
+      </c>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
-      <c r="K22" s="2"/>
+      <c r="K22" s="2" t="s">
+        <v>484</v>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="2" t="s">
@@ -3132,10 +3495,14 @@
       <c r="G23" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="H23" s="2"/>
+      <c r="H23" s="2" t="s">
+        <v>485</v>
+      </c>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
+      <c r="K23" s="2" t="s">
+        <v>486</v>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="2" t="s">
@@ -3159,10 +3526,14 @@
       <c r="G24" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="H24" s="2"/>
+      <c r="H24" s="2" t="s">
+        <v>487</v>
+      </c>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
+      <c r="K24" s="2" t="s">
+        <v>488</v>
+      </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="2" t="s">
@@ -3186,10 +3557,14 @@
       <c r="G25" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="H25" s="2"/>
+      <c r="H25" s="2" t="s">
+        <v>489</v>
+      </c>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
-      <c r="K25" s="2"/>
+      <c r="K25" s="2" t="s">
+        <v>490</v>
+      </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="2" t="s">
@@ -3213,10 +3588,14 @@
       <c r="G26" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="H26" s="2"/>
+      <c r="H26" s="2" t="s">
+        <v>491</v>
+      </c>
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
-      <c r="K26" s="2"/>
+      <c r="K26" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="2" t="s">
@@ -3240,10 +3619,14 @@
       <c r="G27" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="H27" s="2"/>
+      <c r="H27" s="2" t="s">
+        <v>492</v>
+      </c>
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
-      <c r="K27" s="2"/>
+      <c r="K27" s="2" t="s">
+        <v>493</v>
+      </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="2" t="s">
@@ -3267,10 +3650,14 @@
       <c r="G28" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="H28" s="2"/>
+      <c r="H28" s="2" t="s">
+        <v>494</v>
+      </c>
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
-      <c r="K28" s="2"/>
+      <c r="K28" s="2" t="s">
+        <v>495</v>
+      </c>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="2" t="s">
@@ -3294,10 +3681,14 @@
       <c r="G29" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="H29" s="2"/>
+      <c r="H29" s="2" t="s">
+        <v>496</v>
+      </c>
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
-      <c r="K29" s="2"/>
+      <c r="K29" s="2" t="s">
+        <v>497</v>
+      </c>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="2" t="s">
@@ -3321,10 +3712,14 @@
       <c r="G30" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="H30" s="2"/>
+      <c r="H30" s="2" t="s">
+        <v>498</v>
+      </c>
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
-      <c r="K30" s="2"/>
+      <c r="K30" s="2" t="s">
+        <v>499</v>
+      </c>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="2" t="s">
@@ -3348,10 +3743,14 @@
       <c r="G31" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="H31" s="2"/>
+      <c r="H31" s="2" t="s">
+        <v>500</v>
+      </c>
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
-      <c r="K31" s="2"/>
+      <c r="K31" s="2" t="s">
+        <v>501</v>
+      </c>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="2" t="s">
@@ -3429,10 +3828,14 @@
       <c r="G34" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="H34" s="2"/>
+      <c r="H34" s="2" t="s">
+        <v>502</v>
+      </c>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
-      <c r="K34" s="2"/>
+      <c r="K34" s="2" t="s">
+        <v>503</v>
+      </c>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="2" t="s">
@@ -3456,10 +3859,14 @@
       <c r="G35" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="H35" s="2"/>
+      <c r="H35" s="2" t="s">
+        <v>504</v>
+      </c>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
-      <c r="K35" s="2"/>
+      <c r="K35" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="2" t="s">
@@ -3483,10 +3890,14 @@
       <c r="G36" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="H36" s="2"/>
+      <c r="H36" s="2" t="s">
+        <v>505</v>
+      </c>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
-      <c r="K36" s="2"/>
+      <c r="K36" s="2" t="s">
+        <v>506</v>
+      </c>
     </row>
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="2" t="s">
@@ -3510,10 +3921,14 @@
       <c r="G37" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="H37" s="2"/>
+      <c r="H37" s="2" t="s">
+        <v>507</v>
+      </c>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
-      <c r="K37" s="2"/>
+      <c r="K37" s="2" t="s">
+        <v>508</v>
+      </c>
     </row>
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="2" t="s">
@@ -4136,10 +4551,14 @@
       <c r="G2" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="H2" s="2"/>
+      <c r="H2" s="2" t="s">
+        <v>453</v>
+      </c>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
+      <c r="K2" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="2" t="s">
@@ -4163,10 +4582,14 @@
       <c r="G3" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="H3" s="2"/>
+      <c r="H3" s="2" t="s">
+        <v>509</v>
+      </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
+      <c r="K3" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="s">
@@ -4298,10 +4721,14 @@
       <c r="G8" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="H8" s="2"/>
+      <c r="H8" s="2" t="s">
+        <v>510</v>
+      </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
+      <c r="K8" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="2" t="s">
@@ -4789,10 +5216,14 @@
       <c r="G2" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="H2" s="2"/>
+      <c r="H2" s="2" t="s">
+        <v>511</v>
+      </c>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
+      <c r="K2" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="2" t="s">
@@ -4816,10 +5247,14 @@
       <c r="G3" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="H3" s="2"/>
+      <c r="H3" s="2" t="s">
+        <v>512</v>
+      </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
+      <c r="K3" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="s">
@@ -4843,10 +5278,14 @@
       <c r="G4" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="H4" s="2"/>
+      <c r="H4" s="2" t="s">
+        <v>513</v>
+      </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
+      <c r="K4" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="2" t="s">
@@ -4870,10 +5309,14 @@
       <c r="G5" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="H5" s="2"/>
+      <c r="H5" s="2" t="s">
+        <v>514</v>
+      </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
+      <c r="K5" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="2" t="s">
@@ -4897,10 +5340,14 @@
       <c r="G6" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="H6" s="2"/>
+      <c r="H6" s="2" t="s">
+        <v>515</v>
+      </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
+      <c r="K6" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="2" t="s">
@@ -4924,10 +5371,14 @@
       <c r="G7" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="H7" s="2"/>
+      <c r="H7" s="2" t="s">
+        <v>516</v>
+      </c>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
+      <c r="K7" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="2" t="s">
@@ -4951,10 +5402,14 @@
       <c r="G8" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="H8" s="2"/>
+      <c r="H8" s="2" t="s">
+        <v>517</v>
+      </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
+      <c r="K8" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="2" t="s">
@@ -4978,10 +5433,14 @@
       <c r="G9" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="H9" s="2"/>
+      <c r="H9" s="2" t="s">
+        <v>518</v>
+      </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
+      <c r="K9" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="2" t="s">
@@ -5005,10 +5464,14 @@
       <c r="G10" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="H10" s="2"/>
+      <c r="H10" s="2" t="s">
+        <v>519</v>
+      </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
+      <c r="K10" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="2" t="s">
@@ -5491,10 +5954,14 @@
       <c r="G28" s="3" t="s">
         <v>246</v>
       </c>
-      <c r="H28" s="2"/>
+      <c r="H28" s="2" t="s">
+        <v>520</v>
+      </c>
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
-      <c r="K28" s="2"/>
+      <c r="K28" s="2" t="s">
+        <v>521</v>
+      </c>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="2" t="s">
@@ -5518,10 +5985,14 @@
       <c r="G29" s="3" t="s">
         <v>248</v>
       </c>
-      <c r="H29" s="2"/>
+      <c r="H29" s="2" t="s">
+        <v>522</v>
+      </c>
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
-      <c r="K29" s="2"/>
+      <c r="K29" s="2" t="s">
+        <v>523</v>
+      </c>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="2" t="s">
@@ -5653,10 +6124,14 @@
       <c r="G34" s="3" t="s">
         <v>248</v>
       </c>
-      <c r="H34" s="2"/>
+      <c r="H34" s="2" t="s">
+        <v>524</v>
+      </c>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
-      <c r="K34" s="2"/>
+      <c r="K34" s="2" t="s">
+        <v>523</v>
+      </c>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="2" t="s">
@@ -5869,10 +6344,14 @@
       <c r="G42" s="3" t="s">
         <v>269</v>
       </c>
-      <c r="H42" s="2"/>
+      <c r="H42" s="2" t="s">
+        <v>525</v>
+      </c>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
-      <c r="K42" s="2"/>
+      <c r="K42" s="2" t="s">
+        <v>526</v>
+      </c>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="A43" s="2" t="s">
@@ -5896,10 +6375,14 @@
       <c r="G43" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="H43" s="2"/>
+      <c r="H43" s="2" t="s">
+        <v>527</v>
+      </c>
       <c r="I43" s="2"/>
       <c r="J43" s="2"/>
-      <c r="K43" s="2"/>
+      <c r="K43" s="2" t="s">
+        <v>528</v>
+      </c>
     </row>
     <row r="44" ht="30" customHeight="1">
       <c r="A44" s="2" t="s">
@@ -6247,10 +6730,14 @@
       <c r="G56" s="3" t="s">
         <v>248</v>
       </c>
-      <c r="H56" s="2"/>
+      <c r="H56" s="2" t="s">
+        <v>529</v>
+      </c>
       <c r="I56" s="2"/>
       <c r="J56" s="2"/>
-      <c r="K56" s="2"/>
+      <c r="K56" s="2" t="s">
+        <v>523</v>
+      </c>
     </row>
     <row r="57" ht="30" customHeight="1">
       <c r="A57" s="2" t="s">
@@ -6657,10 +7144,14 @@
       <c r="G2" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="H2" s="2"/>
+      <c r="H2" s="2" t="s">
+        <v>530</v>
+      </c>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
+      <c r="K2" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="2" t="s">
@@ -6684,10 +7175,14 @@
       <c r="G3" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="H3" s="2"/>
+      <c r="H3" s="2" t="s">
+        <v>531</v>
+      </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
+      <c r="K3" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="s">
@@ -6711,10 +7206,14 @@
       <c r="G4" s="3" t="s">
         <v>310</v>
       </c>
-      <c r="H4" s="2"/>
+      <c r="H4" s="2" t="s">
+        <v>532</v>
+      </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
+      <c r="K4" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="2" t="s">
@@ -6738,10 +7237,14 @@
       <c r="G5" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="H5" s="2"/>
+      <c r="H5" s="2" t="s">
+        <v>533</v>
+      </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
+      <c r="K5" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="2" t="s">
@@ -6765,10 +7268,14 @@
       <c r="G6" s="3" t="s">
         <v>312</v>
       </c>
-      <c r="H6" s="2"/>
+      <c r="H6" s="2" t="s">
+        <v>534</v>
+      </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
+      <c r="K6" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="2" t="s">
@@ -6792,10 +7299,14 @@
       <c r="G7" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="H7" s="2"/>
+      <c r="H7" s="2" t="s">
+        <v>535</v>
+      </c>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
+      <c r="K7" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="2" t="s">
@@ -7332,10 +7843,14 @@
       <c r="G27" s="3" t="s">
         <v>269</v>
       </c>
-      <c r="H27" s="2"/>
+      <c r="H27" s="2" t="s">
+        <v>536</v>
+      </c>
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
-      <c r="K27" s="2"/>
+      <c r="K27" s="2" t="s">
+        <v>526</v>
+      </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="2" t="s">
@@ -7958,10 +8473,14 @@
       <c r="G2" s="3" t="s">
         <v>379</v>
       </c>
-      <c r="H2" s="2"/>
+      <c r="H2" s="2" t="s">
+        <v>453</v>
+      </c>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
+      <c r="K2" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="2" t="s">
@@ -8012,10 +8531,14 @@
       <c r="G4" s="3" t="s">
         <v>383</v>
       </c>
-      <c r="H4" s="2"/>
+      <c r="H4" s="2" t="s">
+        <v>537</v>
+      </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
+      <c r="K4" s="2" t="s">
+        <v>454</v>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="2" t="s">
@@ -8093,10 +8616,14 @@
       <c r="G7" s="3" t="s">
         <v>269</v>
       </c>
-      <c r="H7" s="2"/>
+      <c r="H7" s="2" t="s">
+        <v>538</v>
+      </c>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
+      <c r="K7" s="2" t="s">
+        <v>539</v>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="2" t="s">
@@ -8876,10 +9403,14 @@
       <c r="G36" s="3" t="s">
         <v>439</v>
       </c>
-      <c r="H36" s="2"/>
+      <c r="H36" s="2" t="s">
+        <v>540</v>
+      </c>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
-      <c r="K36" s="2"/>
+      <c r="K36" s="2" t="s">
+        <v>541</v>
+      </c>
     </row>
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="2" t="s">
@@ -8903,10 +9434,14 @@
       <c r="G37" s="3" t="s">
         <v>441</v>
       </c>
-      <c r="H37" s="2"/>
+      <c r="H37" s="2" t="s">
+        <v>542</v>
+      </c>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
-      <c r="K37" s="2"/>
+      <c r="K37" s="2" t="s">
+        <v>543</v>
+      </c>
     </row>
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="2" t="s">
@@ -8930,10 +9465,14 @@
       <c r="G38" s="3" t="s">
         <v>443</v>
       </c>
-      <c r="H38" s="2"/>
+      <c r="H38" s="2" t="s">
+        <v>544</v>
+      </c>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
-      <c r="K38" s="2"/>
+      <c r="K38" s="2" t="s">
+        <v>545</v>
+      </c>
     </row>
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="2" t="s">

</xml_diff>

<commit_message>
[Liu2017] data dictionary meanings
Fill meaning and notes for all 39 previously-empty rows in the Liu sheet
of Merging/data_dictionaries.xlsx. Sources: Parsing_metadata.qmd,
manuscript (Liu et al. BMT 2017), raw meta_clinical.xlsx, and full scan
of liu_meta_qiime.tsv. Adds fill_liu_meanings.R script.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Merging/data_dictionaries.xlsx
+++ b/Merging/data_dictionaries.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1303" uniqueCount="617">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1376" uniqueCount="688">
   <si>
     <t>column_name</t>
   </si>
@@ -1428,99 +1428,195 @@
     <t>Donor | Patient</t>
   </si>
   <si>
+    <t>Whether the sample is from the transplant recipient or the matched sibling stem cell donor. The study enrolled N=57 recipients and N=22 of their paired HLA-matched sibling donors. Values: Patient | Donor.</t>
+  </si>
+  <si>
+    <t>All clinical outcome columns (disease, GvHD, engraftment, survival) are NA for Donor rows; demographic columns (sex, aborh) are populated for both Donors and Patients.</t>
+  </si>
+  <si>
     <t>40 | 61 | 51 | 69 | 73</t>
   </si>
   <si>
+    <t>Recipient age at transplant. Units: years (integer). Range in data: 22-76. NA for all Donor rows (not collected from donors).</t>
+  </si>
+  <si>
     <t>race</t>
   </si>
   <si>
     <t>asian | white | hispanic | black</t>
   </si>
   <si>
+    <t>Self-reported race of the transplant recipient. Values: white | asian | hispanic | black. NA for Donor rows.</t>
+  </si>
+  <si>
     <t>male | female</t>
   </si>
   <si>
+    <t>Biological sex of the participant (recipient or donor). Values: male | female. Available for both patients and donors.</t>
+  </si>
+  <si>
     <t>aborh</t>
   </si>
   <si>
     <t>A+ | O+ | B+ | A- | O-</t>
   </si>
   <si>
+    <t>ABO blood group and Rh factor of the participant (recipient or donor). Combined blood type string. Values observed: A+ | A- | B+ | B- | O+ | O- | AB+.</t>
+  </si>
+  <si>
     <t>BMI</t>
   </si>
   <si>
     <t>26 | 31 | 34 | 33 | 25</t>
   </si>
   <si>
+    <t>Body mass index of the transplant recipient at or near the time of transplant. Units: kg/m² (integer). Range in data: 18-42. NA for Donor rows.</t>
+  </si>
+  <si>
+    <t>Paper Table 1 defines obesity as BMI &gt;= 30; 18 of 57 recipients (31.6%) were obese.</t>
+  </si>
+  <si>
     <t>TCL | AML | NHL | MDS | ALL</t>
   </si>
   <si>
+    <t>Primary hematologic diagnosis for which the transplant was performed, abbreviated. Values: AML = acute myeloid leukemia; ALL = acute lymphoblastic leukemia; MDS = myelodysplastic syndrome; NHL = non-Hodgkin's lymphoma; CLL = chronic lymphocytic leukemia; TCL = T-cell leukemia/lymphoma; CML = chronic myeloid leukemia; HD = Hodgkin's disease; AA = aplastic anemia. NA for Donor rows.</t>
+  </si>
+  <si>
+    <t>Paper Table 1 lists all nine diagnoses with counts. AML most common (N=24, 42.1%).</t>
+  </si>
+  <si>
     <t>disease_status_at_transplant</t>
   </si>
   <si>
     <t>remission | refractory</t>
   </si>
   <si>
+    <t>Disease status of the recipient at the time of transplant. Values: remission (disease responding to prior treatment) | refractory (disease not responding to treatment; also covers non-malignant diagnoses like AA). NA for Donor rows.</t>
+  </si>
+  <si>
+    <t>Paper Table 1: Remission=28 (49.1%), Refractory/not applicable=29 (50.9%).</t>
+  </si>
+  <si>
     <t>infection_prior_to_transplant</t>
   </si>
   <si>
     <t>no | yes</t>
   </si>
   <si>
+    <t>Whether the recipient had a clinically documented infection in the period prior to transplant. Does not include viral seropositivity (see other_viruses). Values: yes | no. NA for Donor rows.</t>
+  </si>
+  <si>
     <t>other_viruses</t>
   </si>
   <si>
     <t>Missing: not collected | VZV | VZV, HSV | HSV, VZV | HSV, VZV, EBV</t>
   </si>
   <si>
+    <t>Free-text list of prior viral seropositivity or known viral exposures for the recipient, documented before transplant (e.g., VZV, HSV, EBV, CMV, Hepatitis B, Hepatitis C, BK virus, Rhinovirus). Not a structured categorical.</t>
+  </si>
+  <si>
+    <t>UNCERTAIN: the paper does not formally define this field. Values are consistent with seropositive viral exposure history (not necessarily active infection at transplant). The paper adjusts for CMV seropositivity as a statistical covariate (Methods), but there is no separate cmv_status column in liu_meta_qiime.tsv; CMV status is in the raw meta_samples.csv but was excluded in Parsing_metadata.qmd. Checked: paper Methods, Parsing_metadata.qmd.</t>
+  </si>
+  <si>
     <t>gi_history_details</t>
   </si>
   <si>
     <t>partial small bowel resection for obstru | appendectomy, GERD | carcinoid tumor sp bowel resection, GERD | IBS, appendectomy | appendectomy, constipation, polyp, GERD</t>
   </si>
   <si>
+    <t>Free-text description of prior gastrointestinal medical history for the recipient, including past GI surgeries, diagnoses, and conditions (e.g., appendectomy, GERD, cholecystectomy, bowel resection, IBD, Crohn's disease). Not a structured categorical. NA for Donor rows.</t>
+  </si>
+  <si>
+    <t>This was one of the co-morbidity variables associated with recipient microbiome diversity in the paper (Supplementary File 4; P=0.004 for GI/hepatic conditions). 45.6% missing (recipients with no documented GI history record NA, not an empty string).</t>
+  </si>
+  <si>
     <t>donor_source</t>
   </si>
   <si>
     <t>pbsc | cord+cord | marrow</t>
   </si>
   <si>
+    <t>Source of hematopoietic stem cells for the transplant. Values: pbsc = peripheral blood stem cells; marrow = bone marrow; cord+cord = double umbilical cord blood unit transplant. NA for Donor rows.</t>
+  </si>
+  <si>
+    <t>Paper Table 1: PBSC=33 (57.9%), Marrow=3 (5.3%), Cord/Cord=21 (36.8%). For cord+cord transplants, donor_type=cord and no individual living donor was enrolled.</t>
+  </si>
+  <si>
     <t>donor_type</t>
   </si>
   <si>
     <t>related | cord | unrelated</t>
   </si>
   <si>
+    <t>Relationship of the stem cell donor to the recipient. Values: related = HLA-matched related donor (typically sibling); unrelated = HLA-matched unrelated donor (National Marrow Donor Program); cord = umbilical cord blood unit (no living individual donor). NA for Donor rows.</t>
+  </si>
+  <si>
+    <t>For cord+cord transplants (donor_source=cord+cord), donor_type is always cord. The study's sub-cohort with paired donor microbiome samples (N=22) consists exclusively of recipients with related PBSC donors.</t>
+  </si>
+  <si>
     <t>chemotherapy_regimen</t>
   </si>
   <si>
     <t>Flu/Mel | Flu/Cy/Thio/TBI | Flu/Cy/TBI | Flu/TBI | Bu/Cy</t>
   </si>
   <si>
+    <t>Conditioning chemotherapy regimen administered to the recipient before transplant. Drug abbreviations: Flu=fludarabine; Mel=melphalan; TBI=total body irradiation; Bu=busulfan; Cy=cyclophosphamide; Thio=thiotepa; Treo=treosulfan; ATG=anti-thymocyte globulin. Dose notations: TBI(12)=12 Gy, TBI(13G)=13 Gy. Values: Flu/Mel | Flu/TBI | Bu/Cy | Cy/TBI(12) | Flu/Cy/Thio/TBI | Flu/Cy/TBI | Flu/Cy/TBI(13G) | Flu/Treo/TBI | Cy/ATG. NA for Donor rows.</t>
+  </si>
+  <si>
+    <t>Correlated with conditioning_intensity: myeloablative regimens = Bu/Cy or Cy/TBI; reduced-intensity = Flu-based; Cy/ATG = aplastic anemia non-myeloablative conditioning. The paper did not explicitly adjust for this due to collinearity with prophylaxis regimen.</t>
+  </si>
+  <si>
     <t>conditioning_intensity</t>
   </si>
   <si>
     <t>Intermediate intensity | Low intensity | High intensity</t>
   </si>
   <si>
+    <t>Intensity classification of the conditioning regimen. Values: Low intensity (reduced-intensity conditioning, RIC); Intermediate intensity; High intensity (myeloablative conditioning, MAC). NA for Donor rows.</t>
+  </si>
+  <si>
+    <t>Paper Table 1: Low=24 (42.1%), Intermediate=24 (42.1%), High=9 (15.8%).</t>
+  </si>
+  <si>
     <t>cyclosporine</t>
   </si>
   <si>
+    <t>Binary indicator: whether the recipient received cyclosporine as part of GvHD prophylaxis. Values: yes | no. NA for Donor rows.</t>
+  </si>
+  <si>
+    <t>One of five GvHD-prophylaxis indicator columns (cyclosporine, methotrexate, mmf, sirolimus, tacrolimus). These five columns are one-hot expansions of the prophylaxis regimen. The four regimens used in this cohort: cyclosporine/methotrexate (N=2), cyclosporine/MMF (N=21), tacrolimus/methotrexate (N=21), tacrolimus/MMF (N=13) per Table 1. The underlying variable is the two-drug prophylaxis regimen.</t>
+  </si>
+  <si>
     <t>cytogenetics</t>
   </si>
   <si>
     <t>normal | abnormal</t>
   </si>
   <si>
+    <t>Cytogenetic risk classification of the recipient's hematologic malignancy based on karyotype analysis. Values: normal (normal karyotype) | abnormal (abnormal karyotype, higher cytogenetic risk). NA for Donor rows.</t>
+  </si>
+  <si>
+    <t>UNCERTAIN: the paper does not define or describe cytogenetics in the Methods section or Table 1. Column name and binary values (normal/abnormal) are consistent with standard cytogenetic risk classification at diagnosis, but this is not confirmed by the manuscript. Checked: Parsing_metadata.qmd (passed through from meta_clinical.xlsx without annotation), paper Methods, Table 1.</t>
+  </si>
+  <si>
     <t>methotrexate</t>
   </si>
   <si>
     <t>yes | no</t>
   </si>
   <si>
+    <t>Binary indicator: whether the recipient received methotrexate as part of GvHD prophylaxis. Values: yes | no. NA for Donor rows.</t>
+  </si>
+  <si>
+    <t>One of five GvHD-prophylaxis indicator columns. See notes on cyclosporine for the full prophylaxis regimen group.</t>
+  </si>
+  <si>
     <t>mmf</t>
   </si>
   <si>
+    <t>Binary indicator: whether the recipient received mycophenolate mofetil (MMF) as part of GvHD prophylaxis. Values: yes | no. NA for Donor rows.</t>
+  </si>
+  <si>
     <t>sirolimus</t>
   </si>
   <si>
@@ -1530,97 +1626,214 @@
     <t>tacrolimus</t>
   </si>
   <si>
+    <t>Binary indicator: whether the recipient received tacrolimus as part of GvHD prophylaxis. Values: yes | no. NA for Donor rows.</t>
+  </si>
+  <si>
     <t>right_censor_time</t>
   </si>
   <si>
     <t>180 | 365 | 100 | 101 | 61</t>
   </si>
   <si>
+    <t>Administrative follow-up time (right-censoring time) for survival analysis, in days from transplant. For recipients who did not die, this is the duration of documented follow-up (administrative censoring). For deceased recipients, this equals or approximates time_to_death. Time origin: transplant date. Units: days. NA for Donor rows.</t>
+  </si>
+  <si>
+    <t>UNCERTAIN: the paper does not explicitly define right_censor_time. Interpretation as days-from-transplant censoring time is consistent with the paper's Cox proportional hazards model for overall mortality and with values ranging 61-723 days (Table 1 mean follow-up 145 [121] days). One anomalous record (SAMEA4506982) has right_censor_time=365 but time_to_death=345 with deceased=1, suggesting occasional discrepancy. Checked: Parsing_metadata.qmd (passed through from meta_clinical.xlsx), paper Methods.</t>
+  </si>
+  <si>
     <t>deceased</t>
   </si>
   <si>
+    <t>Binary indicator of whether the recipient died during the follow-up period. Values: 0 = alive at last follow-up; 1 = deceased. Time origin: transplant date. NA for Donor rows.</t>
+  </si>
+  <si>
+    <t>Paper Table 1: 18 recipients (31.6%) known to be deceased.</t>
+  </si>
+  <si>
     <t>etiology_of_death</t>
   </si>
   <si>
     <t>Relapse/Resipatory | Relapse | Sepsis/ARDS/GVHD | aGVHD/Infection | Respiratory failure</t>
   </si>
   <si>
+    <t>Free-text cause of death for recipients with deceased=1. Values observed: Relapse; Relapse/Respiratory; Sepsis; Sepsis/ARDS/GVHD; aGVHD/Infection; Respiratory failure; ARDS/Respiratory failure; septic shock. NA if deceased=0, cause unknown, or Donor rows.</t>
+  </si>
+  <si>
+    <t>Causes of death are non-exclusive per Table 1 (one death may count in multiple categories): GvHD=11.1%, Infection/Sepsis=44.4%, Relapse=44.4%, Respiratory failure=22.2%.</t>
+  </si>
+  <si>
     <t>time_to_death</t>
   </si>
   <si>
     <t>61 | 393 | 69 | 250 | 116</t>
   </si>
   <si>
+    <t>Days from transplant to death for recipients with deceased=1. Time origin: transplant date. Event: death. Units: days. NA if deceased=0 or for Donor rows.</t>
+  </si>
+  <si>
+    <t>Paper Table 1: mean time to death 272 (207) days for all recipients, 181 (147) for sub-cohort.</t>
+  </si>
+  <si>
     <t>relapsed</t>
   </si>
   <si>
+    <t>Whether the recipient experienced disease relapse after transplant. Values: yes | no. NA for Donor rows.</t>
+  </si>
+  <si>
+    <t>Paper Table 1: 18 recipients (31.6%) relapsed.</t>
+  </si>
+  <si>
     <t>days_at_relapse</t>
   </si>
   <si>
     <t>367 | 67 | 161 | 159 | 61</t>
   </si>
   <si>
+    <t>Days from transplant to first disease relapse for recipients with relapsed=yes. Time origin: transplant date. Event: disease relapse. Units: days. NA if relapsed=no or Donor rows.</t>
+  </si>
+  <si>
+    <t>83.5% missing (structural: NA for all non-relapsed patients and donors).</t>
+  </si>
+  <si>
     <t>platelet_engrafment</t>
   </si>
   <si>
+    <t>Whether the recipient achieved platelet engraftment after transplant. Values: yes | no. NA for Donor rows.</t>
+  </si>
+  <si>
+    <t>Two recipients did not achieve platelet engraftment (platelet_engrafment=no, days_to_platelet_engrafment=NA): SAMEA4506991 and SAMEA4507002.</t>
+  </si>
+  <si>
     <t>days_to_platelet_engrafment</t>
   </si>
   <si>
     <t>13 | 11 | 27 | 16 | 12</t>
   </si>
   <si>
+    <t>Days from transplant to platelet engraftment. Time origin: transplant date. Event: platelet count &gt;=20,000/μL independent of transfusion support (standard engraftment criterion). Units: days. NA if engraftment not achieved or for Donor rows.</t>
+  </si>
+  <si>
+    <t>Paper Table 1: mean 20.3 (7.37) days for all recipients, 18.5 (6.45) for sub-cohort.</t>
+  </si>
+  <si>
     <t>anc_engrafment</t>
   </si>
   <si>
+    <t>Whether the recipient achieved absolute neutrophil count (ANC) engraftment after transplant. Values: yes | no. NA for Donor rows.</t>
+  </si>
+  <si>
+    <t>Two recipients did not achieve ANC engraftment (SAMEA4506991, SAMEA4507002); same as those lacking platelet engraftment.</t>
+  </si>
+  <si>
     <t>days_to_anc_engrafment</t>
   </si>
   <si>
     <t>15 | 21 | 9 | 22 | 19</t>
   </si>
   <si>
+    <t>Days from transplant to ANC engraftment. Time origin: transplant date. Event: ANC &gt;=500/μL for three consecutive days (standard engraftment criterion). Units: days. NA if engraftment not achieved or for Donor rows.</t>
+  </si>
+  <si>
+    <t>Paper Table 1: mean 20.2 (11.1) days for all recipients, 12.9 (4.41) for sub-cohort.</t>
+  </si>
+  <si>
     <t>agvhd_organ</t>
   </si>
   <si>
     <t>None documented | skin, oral | upper gut | skin, gut | gut</t>
   </si>
   <si>
+    <t>Organ system(s) affected by acute GvHD in the recipient, as a comma-separated free-text list. Values: 'None documented' (no agGVHD observed); or one or more of: skin, gut, upper gut, liver, oral. NA for Donor rows (outcome not applicable).</t>
+  </si>
+  <si>
+    <t>Source variable for two derived columns: agvhd (binary, Parsing_metadata.qmd: agvhd_organ=='None documented' -&gt; 0, else 1) and agvhd_gut (positive if gut/upper gut in organ list). I would keep agvhd_organ as the authoritative source; agvhd and agvhd_gut are derivable from it. Note: 'None documented' (not NA) means no agGVHD was observed; NA means the row is a Donor.</t>
+  </si>
+  <si>
     <t>agvhd_severity</t>
   </si>
   <si>
     <t>no | Grade II | Grade III | Grade I | yes</t>
   </si>
   <si>
+    <t>Severity grade of acute GvHD per the International Bone Marrow Transplant Registry (IBMTR) Severity Index (Rowlings et al., BMT 1997). Values: no (no agGVHD); Grade I (mild); Grade II (moderate); Grade III (severe); Grade IV (life-threatening); yes (agGVHD documented but not formally graded); suspected (clinical suspicion without confirmed diagnosis). NA for Donor rows.</t>
+  </si>
+  <si>
+    <t>UNCERTAIN: values 'yes' and 'suspected' do not map to a standard IBMTR grade. 'Yes' appears when agvhd_organ documents organ involvement but a formal grade is absent; 'suspected' appears in at least one record (SAMEA4507001, agvhd_organ=gut). The paper states grading per IBMTR criteria but these non-standard values are in the raw clinical data. Paper Table 1 reports Glucksberg grades 0/1-2/3-5, which may differ from IBMTR staging terminology. Checked: Parsing_metadata.qmd (passed through from meta_clinical.xlsx), paper Methods.</t>
+  </si>
+  <si>
     <t>agvhd_gut</t>
   </si>
   <si>
     <t>negative | positive</t>
   </si>
   <si>
+    <t>Binary indicator of gut (GI tract) involvement in acute GvHD. Values: positive (gut or upper gut involved) | negative (gut not involved or no agGVHD). NA for Donor rows.</t>
+  </si>
+  <si>
+    <t>Derivable from agvhd_organ: positive corresponds to agvhd_organ containing 'gut' or 'upper gut'. One-hot extraction of gut involvement from the multi-organ agvhd_organ field. Redundant with agvhd_organ; I would keep agvhd_organ as the source. Gut agGVHD was the primary outcome studied in this paper.</t>
+  </si>
+  <si>
     <t>time_to_agvhd</t>
   </si>
   <si>
     <t>28 | 50 | 101 | 37 | 64</t>
   </si>
   <si>
+    <t>Days from transplant to onset of acute GvHD. Time origin: transplant date. Event: first confirmed or clinically suspected agGVHD. Units: days. NA if agvhd=0 (no agGVHD documented) or for Donor rows.</t>
+  </si>
+  <si>
+    <t>63.3% missing (structural: NA for all agGVHD-negative patients and donors).</t>
+  </si>
+  <si>
     <t>cgvhd_severity</t>
   </si>
   <si>
     <t>Stage 1 | Stage 2 | Stage 3</t>
   </si>
   <si>
+    <t>Severity stage of chronic GvHD (cGVHD). Values: none (no cGVHD); Stage 1 (mild); Stage 2 (moderate); Stage 3 (severe). NA for Donor rows or recipients without cGVHD follow-up.</t>
+  </si>
+  <si>
+    <t>UNCERTAIN: staging system (NIH consensus criteria vs. older Shulman/Sullivan clinical staging) is not specified in the paper. Values Stage 1/2/3 are consistent with NIH cGVHD global severity staging (mild/moderate/severe) but could also reflect older staging. Chronic GvHD is not the primary outcome and its grading is not described in the Methods. Checked: Parsing_metadata.qmd, paper Methods. 75.9% missing.</t>
+  </si>
+  <si>
     <t>time_to_cgvhd</t>
   </si>
   <si>
+    <t>Days from transplant to onset of chronic GvHD. Time origin: transplant date. Event: first confirmed cGVHD. Units: days. NA if cgvhd_severity=none, missing cGVHD data, or Donor rows.</t>
+  </si>
+  <si>
+    <t>62.0% missing (structural for patients without cGVHD and donors).</t>
+  </si>
+  <si>
     <t>infection_duringafter_transplant</t>
   </si>
   <si>
     <t>diverticulitis, neutropenic fever, oral  | oral candida, VRE | neutropenic fever, C difficile colitis,  | Enterococcus UTI | oral candida, rhinovirus</t>
   </si>
   <si>
+    <t>Free-text list of clinically significant infections occurring during or after the transplant course. Records organism names and infection types (e.g., 'C difficile, CMV viremia, VRE bacteremia, pneumonia'). NA if no documented infections or for Donor rows.</t>
+  </si>
+  <si>
+    <t>UNCERTAIN: the distinction between infection_duringafter_transplant and infection_details is not defined in the paper or Parsing_metadata.qmd. Both are free-text infection fields; in the data, this column appears to capture the primary infection list while infection_details captures supplementary or ancillary infections, but the split is inconsistent across records (some rows have data in one field only, some in both, with no clear rule). Checked: Parsing_metadata.qmd, paper Methods. I would treat this column as primary and infection_details as supplementary.</t>
+  </si>
+  <si>
     <t>infection_details</t>
   </si>
   <si>
     <t>perifacial abscess | EBV | Leuconostoc bacteremia, sinusitis | C difficile, recurrence | aspergillus pneumonia/sinusitis</t>
+  </si>
+  <si>
+    <t>Additional free-text details about post-transplant infections, supplementing infection_duringafter_transplant. May contain secondary organisms, additional diagnoses, or context not captured in the primary infection field.</t>
+  </si>
+  <si>
+    <t>UNCERTAIN: distinction from infection_duringafter_transplant is not defined. See notes on infection_duringafter_transplant. The two columns are partially redundant: 41.8% and 63.3% missing respectively, with different subsets of patients contributing data to each. Checked: Parsing_metadata.qmd, paper Methods.</t>
+  </si>
+  <si>
+    <t>Binary indicator of any acute GvHD occurrence, derived in Parsing_metadata.qmd from agvhd_organ. Values: 0 = no agGVHD (agvhd_organ == 'None documented'); 1 = agGVHD documented in at least one organ system. NA for Donor rows (agvhd_organ is NA).</t>
+  </si>
+  <si>
+    <t>Derived column: case_when(is.na(agvhd_organ) ~ NA, agvhd_organ == 'None documented' ~ 0, TRUE ~ 1). Redundant with agvhd_organ (source) and partially with agvhd_gut (binary for gut involvement only). I would keep agvhd as the primary binary endpoint for analysis (it is the outcome in the paper's logistic regression models) and agvhd_organ for organ-level detail. See agvhd_organ notes for the full redundancy group (agvhd_organ, agvhd, agvhd_gut).</t>
   </si>
   <si>
     <t>SRR22325945 | SRR22325944 | SRR22325892 | SRR22325891 | SRR22325890</t>
@@ -7084,6 +7297,12 @@
       <c r="G8" t="s">
         <v>468</v>
       </c>
+      <c r="H8" t="s">
+        <v>469</v>
+      </c>
+      <c r="K8" t="s">
+        <v>470</v>
+      </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" t="s">
@@ -7105,12 +7324,15 @@
         <v>27</v>
       </c>
       <c r="G9" t="s">
-        <v>469</v>
+        <v>471</v>
+      </c>
+      <c r="H9" t="s">
+        <v>472</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="B10">
         <v>4</v>
@@ -7128,7 +7350,10 @@
         <v>32</v>
       </c>
       <c r="G10" t="s">
-        <v>471</v>
+        <v>474</v>
+      </c>
+      <c r="H10" t="s">
+        <v>475</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -7151,12 +7376,15 @@
         <v>32</v>
       </c>
       <c r="G11" t="s">
-        <v>472</v>
+        <v>476</v>
+      </c>
+      <c r="H11" t="s">
+        <v>477</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" t="s">
-        <v>473</v>
+        <v>478</v>
       </c>
       <c r="B12">
         <v>7</v>
@@ -7174,12 +7402,15 @@
         <v>32</v>
       </c>
       <c r="G12" t="s">
-        <v>474</v>
+        <v>479</v>
+      </c>
+      <c r="H12" t="s">
+        <v>480</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>475</v>
+        <v>481</v>
       </c>
       <c r="B13">
         <v>20</v>
@@ -7197,7 +7428,13 @@
         <v>27</v>
       </c>
       <c r="G13" t="s">
-        <v>476</v>
+        <v>482</v>
+      </c>
+      <c r="H13" t="s">
+        <v>483</v>
+      </c>
+      <c r="K13" t="s">
+        <v>484</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -7220,12 +7457,18 @@
         <v>32</v>
       </c>
       <c r="G14" t="s">
-        <v>477</v>
+        <v>485</v>
+      </c>
+      <c r="H14" t="s">
+        <v>486</v>
+      </c>
+      <c r="K14" t="s">
+        <v>487</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" t="s">
-        <v>478</v>
+        <v>488</v>
       </c>
       <c r="B15">
         <v>2</v>
@@ -7243,12 +7486,18 @@
         <v>32</v>
       </c>
       <c r="G15" t="s">
-        <v>479</v>
+        <v>489</v>
+      </c>
+      <c r="H15" t="s">
+        <v>490</v>
+      </c>
+      <c r="K15" t="s">
+        <v>491</v>
       </c>
     </row>
     <row r="16" spans="1:11">
       <c r="A16" t="s">
-        <v>480</v>
+        <v>492</v>
       </c>
       <c r="B16">
         <v>2</v>
@@ -7266,12 +7515,15 @@
         <v>60</v>
       </c>
       <c r="G16" t="s">
-        <v>481</v>
+        <v>493</v>
+      </c>
+      <c r="H16" t="s">
+        <v>494</v>
       </c>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" t="s">
-        <v>482</v>
+        <v>495</v>
       </c>
       <c r="B17">
         <v>18</v>
@@ -7289,12 +7541,18 @@
         <v>32</v>
       </c>
       <c r="G17" t="s">
-        <v>483</v>
+        <v>496</v>
+      </c>
+      <c r="H17" t="s">
+        <v>497</v>
+      </c>
+      <c r="K17" t="s">
+        <v>498</v>
       </c>
     </row>
     <row r="18" spans="1:11">
       <c r="A18" t="s">
-        <v>484</v>
+        <v>499</v>
       </c>
       <c r="B18">
         <v>33</v>
@@ -7312,12 +7570,18 @@
         <v>32</v>
       </c>
       <c r="G18" t="s">
-        <v>485</v>
+        <v>500</v>
+      </c>
+      <c r="H18" t="s">
+        <v>501</v>
+      </c>
+      <c r="K18" t="s">
+        <v>502</v>
       </c>
     </row>
     <row r="19" spans="1:11">
       <c r="A19" t="s">
-        <v>486</v>
+        <v>503</v>
       </c>
       <c r="B19">
         <v>3</v>
@@ -7335,12 +7599,18 @@
         <v>32</v>
       </c>
       <c r="G19" t="s">
-        <v>487</v>
+        <v>504</v>
+      </c>
+      <c r="H19" t="s">
+        <v>505</v>
+      </c>
+      <c r="K19" t="s">
+        <v>506</v>
       </c>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" t="s">
-        <v>488</v>
+        <v>507</v>
       </c>
       <c r="B20">
         <v>3</v>
@@ -7358,12 +7628,18 @@
         <v>32</v>
       </c>
       <c r="G20" t="s">
-        <v>489</v>
+        <v>508</v>
+      </c>
+      <c r="H20" t="s">
+        <v>509</v>
+      </c>
+      <c r="K20" t="s">
+        <v>510</v>
       </c>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" t="s">
-        <v>490</v>
+        <v>511</v>
       </c>
       <c r="B21">
         <v>9</v>
@@ -7381,12 +7657,18 @@
         <v>32</v>
       </c>
       <c r="G21" t="s">
-        <v>491</v>
+        <v>512</v>
+      </c>
+      <c r="H21" t="s">
+        <v>513</v>
+      </c>
+      <c r="K21" t="s">
+        <v>514</v>
       </c>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" t="s">
-        <v>492</v>
+        <v>515</v>
       </c>
       <c r="B22">
         <v>3</v>
@@ -7404,12 +7686,18 @@
         <v>32</v>
       </c>
       <c r="G22" t="s">
-        <v>493</v>
+        <v>516</v>
+      </c>
+      <c r="H22" t="s">
+        <v>517</v>
+      </c>
+      <c r="K22" t="s">
+        <v>518</v>
       </c>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" t="s">
-        <v>494</v>
+        <v>519</v>
       </c>
       <c r="B23">
         <v>2</v>
@@ -7427,12 +7715,18 @@
         <v>60</v>
       </c>
       <c r="G23" t="s">
-        <v>481</v>
+        <v>493</v>
+      </c>
+      <c r="H23" t="s">
+        <v>520</v>
+      </c>
+      <c r="K23" t="s">
+        <v>521</v>
       </c>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" t="s">
-        <v>495</v>
+        <v>522</v>
       </c>
       <c r="B24">
         <v>2</v>
@@ -7450,12 +7744,18 @@
         <v>32</v>
       </c>
       <c r="G24" t="s">
-        <v>496</v>
+        <v>523</v>
+      </c>
+      <c r="H24" t="s">
+        <v>524</v>
+      </c>
+      <c r="K24" t="s">
+        <v>525</v>
       </c>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" t="s">
-        <v>497</v>
+        <v>526</v>
       </c>
       <c r="B25">
         <v>2</v>
@@ -7473,12 +7773,18 @@
         <v>60</v>
       </c>
       <c r="G25" t="s">
-        <v>498</v>
+        <v>527</v>
+      </c>
+      <c r="H25" t="s">
+        <v>528</v>
+      </c>
+      <c r="K25" t="s">
+        <v>529</v>
       </c>
     </row>
     <row r="26" spans="1:11">
       <c r="A26" t="s">
-        <v>499</v>
+        <v>530</v>
       </c>
       <c r="B26">
         <v>2</v>
@@ -7496,12 +7802,18 @@
         <v>60</v>
       </c>
       <c r="G26" t="s">
-        <v>481</v>
+        <v>493</v>
+      </c>
+      <c r="H26" t="s">
+        <v>531</v>
+      </c>
+      <c r="K26" t="s">
+        <v>529</v>
       </c>
     </row>
     <row r="27" spans="1:11">
       <c r="A27" t="s">
-        <v>500</v>
+        <v>532</v>
       </c>
       <c r="B27">
         <v>1</v>
@@ -7522,7 +7834,7 @@
         <v>412</v>
       </c>
       <c r="H27" t="s">
-        <v>501</v>
+        <v>533</v>
       </c>
       <c r="K27" t="s">
         <v>414</v>
@@ -7530,7 +7842,7 @@
     </row>
     <row r="28" spans="1:11">
       <c r="A28" t="s">
-        <v>502</v>
+        <v>534</v>
       </c>
       <c r="B28">
         <v>2</v>
@@ -7548,12 +7860,18 @@
         <v>60</v>
       </c>
       <c r="G28" t="s">
-        <v>498</v>
+        <v>527</v>
+      </c>
+      <c r="H28" t="s">
+        <v>535</v>
+      </c>
+      <c r="K28" t="s">
+        <v>529</v>
       </c>
     </row>
     <row r="29" spans="1:11">
       <c r="A29" t="s">
-        <v>503</v>
+        <v>536</v>
       </c>
       <c r="B29">
         <v>29</v>
@@ -7571,12 +7889,18 @@
         <v>27</v>
       </c>
       <c r="G29" t="s">
-        <v>504</v>
+        <v>537</v>
+      </c>
+      <c r="H29" t="s">
+        <v>538</v>
+      </c>
+      <c r="K29" t="s">
+        <v>539</v>
       </c>
     </row>
     <row r="30" spans="1:11">
       <c r="A30" t="s">
-        <v>505</v>
+        <v>540</v>
       </c>
       <c r="B30">
         <v>2</v>
@@ -7596,10 +7920,16 @@
       <c r="G30" t="s">
         <v>276</v>
       </c>
+      <c r="H30" t="s">
+        <v>541</v>
+      </c>
+      <c r="K30" t="s">
+        <v>542</v>
+      </c>
     </row>
     <row r="31" spans="1:11">
       <c r="A31" t="s">
-        <v>506</v>
+        <v>543</v>
       </c>
       <c r="B31">
         <v>8</v>
@@ -7617,12 +7947,18 @@
         <v>32</v>
       </c>
       <c r="G31" t="s">
-        <v>507</v>
+        <v>544</v>
+      </c>
+      <c r="H31" t="s">
+        <v>545</v>
+      </c>
+      <c r="K31" t="s">
+        <v>546</v>
       </c>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" t="s">
-        <v>508</v>
+        <v>547</v>
       </c>
       <c r="B32">
         <v>17</v>
@@ -7640,12 +7976,18 @@
         <v>27</v>
       </c>
       <c r="G32" t="s">
-        <v>509</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7">
+        <v>548</v>
+      </c>
+      <c r="H32" t="s">
+        <v>549</v>
+      </c>
+      <c r="K32" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11">
       <c r="A33" t="s">
-        <v>510</v>
+        <v>551</v>
       </c>
       <c r="B33">
         <v>2</v>
@@ -7663,12 +8005,18 @@
         <v>60</v>
       </c>
       <c r="G33" t="s">
-        <v>481</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7">
+        <v>493</v>
+      </c>
+      <c r="H33" t="s">
+        <v>552</v>
+      </c>
+      <c r="K33" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11">
       <c r="A34" t="s">
-        <v>511</v>
+        <v>554</v>
       </c>
       <c r="B34">
         <v>13</v>
@@ -7686,12 +8034,18 @@
         <v>27</v>
       </c>
       <c r="G34" t="s">
-        <v>512</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7">
+        <v>555</v>
+      </c>
+      <c r="H34" t="s">
+        <v>556</v>
+      </c>
+      <c r="K34" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11">
       <c r="A35" t="s">
-        <v>513</v>
+        <v>558</v>
       </c>
       <c r="B35">
         <v>2</v>
@@ -7709,12 +8063,18 @@
         <v>60</v>
       </c>
       <c r="G35" t="s">
-        <v>498</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7">
+        <v>527</v>
+      </c>
+      <c r="H35" t="s">
+        <v>559</v>
+      </c>
+      <c r="K35" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11">
       <c r="A36" t="s">
-        <v>514</v>
+        <v>561</v>
       </c>
       <c r="B36">
         <v>24</v>
@@ -7732,12 +8092,18 @@
         <v>27</v>
       </c>
       <c r="G36" t="s">
-        <v>515</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7">
+        <v>562</v>
+      </c>
+      <c r="H36" t="s">
+        <v>563</v>
+      </c>
+      <c r="K36" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11">
       <c r="A37" t="s">
-        <v>516</v>
+        <v>565</v>
       </c>
       <c r="B37">
         <v>2</v>
@@ -7755,12 +8121,18 @@
         <v>60</v>
       </c>
       <c r="G37" t="s">
-        <v>498</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7">
+        <v>527</v>
+      </c>
+      <c r="H37" t="s">
+        <v>566</v>
+      </c>
+      <c r="K37" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11">
       <c r="A38" t="s">
-        <v>517</v>
+        <v>568</v>
       </c>
       <c r="B38">
         <v>21</v>
@@ -7778,12 +8150,18 @@
         <v>27</v>
       </c>
       <c r="G38" t="s">
-        <v>518</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7">
+        <v>569</v>
+      </c>
+      <c r="H38" t="s">
+        <v>570</v>
+      </c>
+      <c r="K38" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11">
       <c r="A39" t="s">
-        <v>519</v>
+        <v>572</v>
       </c>
       <c r="B39">
         <v>10</v>
@@ -7801,12 +8179,18 @@
         <v>32</v>
       </c>
       <c r="G39" t="s">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7">
+        <v>573</v>
+      </c>
+      <c r="H39" t="s">
+        <v>574</v>
+      </c>
+      <c r="K39" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11">
       <c r="A40" t="s">
-        <v>521</v>
+        <v>576</v>
       </c>
       <c r="B40">
         <v>7</v>
@@ -7824,12 +8208,18 @@
         <v>32</v>
       </c>
       <c r="G40" t="s">
-        <v>522</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7">
+        <v>577</v>
+      </c>
+      <c r="H40" t="s">
+        <v>578</v>
+      </c>
+      <c r="K40" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11">
       <c r="A41" t="s">
-        <v>523</v>
+        <v>580</v>
       </c>
       <c r="B41">
         <v>2</v>
@@ -7847,12 +8237,18 @@
         <v>32</v>
       </c>
       <c r="G41" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7">
+        <v>581</v>
+      </c>
+      <c r="H41" t="s">
+        <v>582</v>
+      </c>
+      <c r="K41" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11">
       <c r="A42" t="s">
-        <v>525</v>
+        <v>584</v>
       </c>
       <c r="B42">
         <v>24</v>
@@ -7870,12 +8266,18 @@
         <v>27</v>
       </c>
       <c r="G42" t="s">
-        <v>526</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7">
+        <v>585</v>
+      </c>
+      <c r="H42" t="s">
+        <v>586</v>
+      </c>
+      <c r="K42" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11">
       <c r="A43" t="s">
-        <v>527</v>
+        <v>588</v>
       </c>
       <c r="B43">
         <v>3</v>
@@ -7893,12 +8295,18 @@
         <v>32</v>
       </c>
       <c r="G43" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7">
+        <v>589</v>
+      </c>
+      <c r="H43" t="s">
+        <v>590</v>
+      </c>
+      <c r="K43" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11">
       <c r="A44" t="s">
-        <v>529</v>
+        <v>592</v>
       </c>
       <c r="B44">
         <v>25</v>
@@ -7916,12 +8324,18 @@
         <v>27</v>
       </c>
       <c r="G44" t="s">
-        <v>526</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7">
+        <v>585</v>
+      </c>
+      <c r="H44" t="s">
+        <v>593</v>
+      </c>
+      <c r="K44" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11">
       <c r="A45" t="s">
-        <v>530</v>
+        <v>595</v>
       </c>
       <c r="B45">
         <v>45</v>
@@ -7939,12 +8353,18 @@
         <v>13</v>
       </c>
       <c r="G45" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7">
+        <v>596</v>
+      </c>
+      <c r="H45" t="s">
+        <v>597</v>
+      </c>
+      <c r="K45" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11">
       <c r="A46" t="s">
-        <v>532</v>
+        <v>599</v>
       </c>
       <c r="B46">
         <v>27</v>
@@ -7962,10 +8382,16 @@
         <v>13</v>
       </c>
       <c r="G46" t="s">
-        <v>533</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7">
+        <v>600</v>
+      </c>
+      <c r="H46" t="s">
+        <v>601</v>
+      </c>
+      <c r="K46" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11">
       <c r="A47" t="s">
         <v>393</v>
       </c>
@@ -7986,6 +8412,12 @@
       </c>
       <c r="G47" t="s">
         <v>276</v>
+      </c>
+      <c r="H47" t="s">
+        <v>603</v>
+      </c>
+      <c r="K47" t="s">
+        <v>604</v>
       </c>
     </row>
   </sheetData>
@@ -8053,7 +8485,7 @@
         <v>13</v>
       </c>
       <c r="G2" t="s">
-        <v>534</v>
+        <v>605</v>
       </c>
       <c r="H2" t="s">
         <v>15</v>
@@ -8064,7 +8496,7 @@
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>535</v>
+        <v>606</v>
       </c>
       <c r="B3">
         <v>50</v>
@@ -8082,12 +8514,12 @@
         <v>32</v>
       </c>
       <c r="G3" t="s">
-        <v>536</v>
+        <v>607</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
-        <v>537</v>
+        <v>608</v>
       </c>
       <c r="B4">
         <v>118</v>
@@ -8105,10 +8537,10 @@
         <v>13</v>
       </c>
       <c r="G4" t="s">
-        <v>538</v>
+        <v>609</v>
       </c>
       <c r="H4" t="s">
-        <v>539</v>
+        <v>610</v>
       </c>
       <c r="K4" t="s">
         <v>16</v>
@@ -8116,7 +8548,7 @@
     </row>
     <row r="5" spans="1:11">
       <c r="A5" t="s">
-        <v>540</v>
+        <v>611</v>
       </c>
       <c r="B5">
         <v>50</v>
@@ -8134,12 +8566,12 @@
         <v>32</v>
       </c>
       <c r="G5" t="s">
-        <v>541</v>
+        <v>612</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>542</v>
+        <v>613</v>
       </c>
       <c r="B6">
         <v>82</v>
@@ -8154,15 +8586,15 @@
         <v>26</v>
       </c>
       <c r="F6" t="s">
-        <v>543</v>
+        <v>614</v>
       </c>
       <c r="G6" t="s">
-        <v>544</v>
+        <v>615</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>545</v>
+        <v>616</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -8183,15 +8615,15 @@
         <v>412</v>
       </c>
       <c r="H7" t="s">
-        <v>546</v>
+        <v>617</v>
       </c>
       <c r="K7" t="s">
-        <v>547</v>
+        <v>618</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>548</v>
+        <v>619</v>
       </c>
       <c r="B8">
         <v>46</v>
@@ -8206,15 +8638,15 @@
         <v>26</v>
       </c>
       <c r="F8" t="s">
-        <v>543</v>
+        <v>614</v>
       </c>
       <c r="G8" t="s">
-        <v>549</v>
+        <v>620</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>550</v>
+        <v>621</v>
       </c>
       <c r="B9">
         <v>47</v>
@@ -8229,15 +8661,15 @@
         <v>26</v>
       </c>
       <c r="F9" t="s">
-        <v>543</v>
+        <v>614</v>
       </c>
       <c r="G9" t="s">
-        <v>551</v>
+        <v>622</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>552</v>
+        <v>623</v>
       </c>
       <c r="B10">
         <v>3</v>
@@ -8255,12 +8687,12 @@
         <v>32</v>
       </c>
       <c r="G10" t="s">
-        <v>553</v>
+        <v>624</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" t="s">
-        <v>554</v>
+        <v>625</v>
       </c>
       <c r="B11">
         <v>3</v>
@@ -8278,12 +8710,12 @@
         <v>32</v>
       </c>
       <c r="G11" t="s">
-        <v>555</v>
+        <v>626</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" t="s">
-        <v>556</v>
+        <v>627</v>
       </c>
       <c r="B12">
         <v>3</v>
@@ -8301,12 +8733,12 @@
         <v>32</v>
       </c>
       <c r="G12" t="s">
-        <v>557</v>
+        <v>628</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>558</v>
+        <v>629</v>
       </c>
       <c r="B13">
         <v>2</v>
@@ -8324,12 +8756,12 @@
         <v>32</v>
       </c>
       <c r="G13" t="s">
-        <v>559</v>
+        <v>630</v>
       </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" t="s">
-        <v>488</v>
+        <v>507</v>
       </c>
       <c r="B14">
         <v>2</v>
@@ -8347,12 +8779,12 @@
         <v>32</v>
       </c>
       <c r="G14" t="s">
-        <v>560</v>
+        <v>631</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" t="s">
-        <v>561</v>
+        <v>632</v>
       </c>
       <c r="B15">
         <v>3</v>
@@ -8370,7 +8802,7 @@
         <v>32</v>
       </c>
       <c r="G15" t="s">
-        <v>562</v>
+        <v>633</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -8398,7 +8830,7 @@
     </row>
     <row r="17" spans="1:7">
       <c r="A17" t="s">
-        <v>563</v>
+        <v>634</v>
       </c>
       <c r="B17">
         <v>3</v>
@@ -8416,12 +8848,12 @@
         <v>27</v>
       </c>
       <c r="G17" t="s">
-        <v>564</v>
+        <v>635</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" t="s">
-        <v>565</v>
+        <v>636</v>
       </c>
       <c r="B18">
         <v>30</v>
@@ -8436,10 +8868,10 @@
         <v>26</v>
       </c>
       <c r="F18" t="s">
-        <v>543</v>
+        <v>614</v>
       </c>
       <c r="G18" t="s">
-        <v>566</v>
+        <v>637</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -8462,12 +8894,12 @@
         <v>27</v>
       </c>
       <c r="G19" t="s">
-        <v>567</v>
+        <v>638</v>
       </c>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" t="s">
-        <v>568</v>
+        <v>639</v>
       </c>
       <c r="B20">
         <v>2</v>
@@ -8490,7 +8922,7 @@
     </row>
     <row r="21" spans="1:7">
       <c r="A21" t="s">
-        <v>569</v>
+        <v>640</v>
       </c>
       <c r="B21">
         <v>18</v>
@@ -8505,15 +8937,15 @@
         <v>26</v>
       </c>
       <c r="F21" t="s">
-        <v>543</v>
+        <v>614</v>
       </c>
       <c r="G21" t="s">
-        <v>570</v>
+        <v>641</v>
       </c>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" t="s">
-        <v>571</v>
+        <v>642</v>
       </c>
       <c r="B22">
         <v>17</v>
@@ -8528,15 +8960,15 @@
         <v>26</v>
       </c>
       <c r="F22" t="s">
-        <v>543</v>
+        <v>614</v>
       </c>
       <c r="G22" t="s">
-        <v>572</v>
+        <v>643</v>
       </c>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" t="s">
-        <v>573</v>
+        <v>644</v>
       </c>
       <c r="B23">
         <v>30</v>
@@ -8551,15 +8983,15 @@
         <v>26</v>
       </c>
       <c r="F23" t="s">
-        <v>543</v>
+        <v>614</v>
       </c>
       <c r="G23" t="s">
-        <v>574</v>
+        <v>645</v>
       </c>
     </row>
     <row r="24" spans="1:7">
       <c r="A24" t="s">
-        <v>575</v>
+        <v>646</v>
       </c>
       <c r="B24">
         <v>49</v>
@@ -8574,15 +9006,15 @@
         <v>26</v>
       </c>
       <c r="F24" t="s">
-        <v>543</v>
+        <v>614</v>
       </c>
       <c r="G24" t="s">
-        <v>576</v>
+        <v>647</v>
       </c>
     </row>
     <row r="25" spans="1:7">
       <c r="A25" t="s">
-        <v>577</v>
+        <v>648</v>
       </c>
       <c r="B25">
         <v>18</v>
@@ -8597,10 +9029,10 @@
         <v>26</v>
       </c>
       <c r="F25" t="s">
-        <v>543</v>
+        <v>614</v>
       </c>
       <c r="G25" t="s">
-        <v>572</v>
+        <v>643</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -8623,12 +9055,12 @@
         <v>36</v>
       </c>
       <c r="G26" t="s">
-        <v>578</v>
+        <v>649</v>
       </c>
     </row>
     <row r="27" spans="1:7">
       <c r="A27" t="s">
-        <v>579</v>
+        <v>650</v>
       </c>
       <c r="B27">
         <v>2</v>
@@ -8651,7 +9083,7 @@
     </row>
     <row r="28" spans="1:7">
       <c r="A28" t="s">
-        <v>580</v>
+        <v>651</v>
       </c>
       <c r="B28">
         <v>8</v>
@@ -8669,12 +9101,12 @@
         <v>32</v>
       </c>
       <c r="G28" t="s">
-        <v>581</v>
+        <v>652</v>
       </c>
     </row>
     <row r="29" spans="1:7">
       <c r="A29" t="s">
-        <v>582</v>
+        <v>653</v>
       </c>
       <c r="B29">
         <v>11</v>
@@ -8692,12 +9124,12 @@
         <v>32</v>
       </c>
       <c r="G29" t="s">
-        <v>583</v>
+        <v>654</v>
       </c>
     </row>
     <row r="30" spans="1:7">
       <c r="A30" t="s">
-        <v>584</v>
+        <v>655</v>
       </c>
       <c r="B30">
         <v>7</v>
@@ -8715,12 +9147,12 @@
         <v>32</v>
       </c>
       <c r="G30" t="s">
-        <v>585</v>
+        <v>656</v>
       </c>
     </row>
     <row r="31" spans="1:7">
       <c r="A31" t="s">
-        <v>586</v>
+        <v>657</v>
       </c>
       <c r="B31">
         <v>2</v>
@@ -8738,12 +9170,12 @@
         <v>32</v>
       </c>
       <c r="G31" t="s">
-        <v>587</v>
+        <v>658</v>
       </c>
     </row>
     <row r="32" spans="1:7">
       <c r="A32" t="s">
-        <v>588</v>
+        <v>659</v>
       </c>
       <c r="B32">
         <v>4</v>
@@ -8761,12 +9193,12 @@
         <v>32</v>
       </c>
       <c r="G32" t="s">
-        <v>589</v>
+        <v>660</v>
       </c>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" t="s">
-        <v>590</v>
+        <v>661</v>
       </c>
       <c r="B33">
         <v>3</v>
@@ -8784,12 +9216,12 @@
         <v>32</v>
       </c>
       <c r="G33" t="s">
-        <v>591</v>
+        <v>662</v>
       </c>
     </row>
     <row r="34" spans="1:11">
       <c r="A34" t="s">
-        <v>592</v>
+        <v>663</v>
       </c>
       <c r="B34">
         <v>40</v>
@@ -8807,12 +9239,12 @@
         <v>27</v>
       </c>
       <c r="G34" t="s">
-        <v>593</v>
+        <v>664</v>
       </c>
     </row>
     <row r="35" spans="1:11">
       <c r="A35" t="s">
-        <v>594</v>
+        <v>665</v>
       </c>
       <c r="B35">
         <v>37</v>
@@ -8830,12 +9262,12 @@
         <v>27</v>
       </c>
       <c r="G35" t="s">
-        <v>595</v>
+        <v>666</v>
       </c>
     </row>
     <row r="36" spans="1:11">
       <c r="A36" t="s">
-        <v>596</v>
+        <v>667</v>
       </c>
       <c r="B36">
         <v>1</v>
@@ -8853,18 +9285,18 @@
         <v>32</v>
       </c>
       <c r="G36" t="s">
-        <v>597</v>
+        <v>668</v>
       </c>
       <c r="H36" t="s">
-        <v>598</v>
+        <v>669</v>
       </c>
       <c r="K36" t="s">
-        <v>599</v>
+        <v>670</v>
       </c>
     </row>
     <row r="37" spans="1:11">
       <c r="A37" t="s">
-        <v>600</v>
+        <v>671</v>
       </c>
       <c r="B37">
         <v>1</v>
@@ -8879,21 +9311,21 @@
         <v>115</v>
       </c>
       <c r="F37" t="s">
-        <v>543</v>
+        <v>614</v>
       </c>
       <c r="G37" t="s">
-        <v>601</v>
+        <v>672</v>
       </c>
       <c r="H37" t="s">
-        <v>602</v>
+        <v>673</v>
       </c>
       <c r="K37" t="s">
-        <v>603</v>
+        <v>674</v>
       </c>
     </row>
     <row r="38" spans="1:11">
       <c r="A38" t="s">
-        <v>604</v>
+        <v>675</v>
       </c>
       <c r="B38">
         <v>1</v>
@@ -8911,18 +9343,18 @@
         <v>60</v>
       </c>
       <c r="G38" t="s">
-        <v>605</v>
+        <v>676</v>
       </c>
       <c r="H38" t="s">
-        <v>606</v>
+        <v>677</v>
       </c>
       <c r="K38" t="s">
-        <v>607</v>
+        <v>678</v>
       </c>
     </row>
     <row r="39" spans="1:11">
       <c r="A39" t="s">
-        <v>608</v>
+        <v>679</v>
       </c>
       <c r="B39">
         <v>28</v>
@@ -8937,15 +9369,15 @@
         <v>26</v>
       </c>
       <c r="F39" t="s">
-        <v>543</v>
+        <v>614</v>
       </c>
       <c r="G39" t="s">
-        <v>609</v>
+        <v>680</v>
       </c>
     </row>
     <row r="40" spans="1:11">
       <c r="A40" t="s">
-        <v>610</v>
+        <v>681</v>
       </c>
       <c r="B40">
         <v>3</v>
@@ -8963,12 +9395,12 @@
         <v>32</v>
       </c>
       <c r="G40" t="s">
-        <v>611</v>
+        <v>682</v>
       </c>
     </row>
     <row r="41" spans="1:11">
       <c r="A41" t="s">
-        <v>612</v>
+        <v>683</v>
       </c>
       <c r="B41">
         <v>2</v>
@@ -8986,12 +9418,12 @@
         <v>32</v>
       </c>
       <c r="G41" t="s">
-        <v>613</v>
+        <v>684</v>
       </c>
     </row>
     <row r="42" spans="1:11">
       <c r="A42" t="s">
-        <v>614</v>
+        <v>685</v>
       </c>
       <c r="B42">
         <v>2</v>
@@ -9009,12 +9441,12 @@
         <v>32</v>
       </c>
       <c r="G42" t="s">
-        <v>613</v>
+        <v>684</v>
       </c>
     </row>
     <row r="43" spans="1:11">
       <c r="A43" t="s">
-        <v>615</v>
+        <v>686</v>
       </c>
       <c r="B43">
         <v>4</v>
@@ -9032,7 +9464,7 @@
         <v>32</v>
       </c>
       <c r="G43" t="s">
-        <v>616</v>
+        <v>687</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[DAmico] data dictionary meanings
Fill meaning (and notes where applicable) for all 26 previously-empty rows
in the DAmico sheet of data_dictionaries.xlsx. Covers SRA administrative
columns, derived parsing columns (second_num, Timepoint, Patient), and all
clinical columns from meta_clinical.csv (Nutritional_Regimen, Sex, Age,
Diagnosis, Donor_Type, Stem_cell_source, Conditioning_regimen, PMN_day,
PLT_over_20000_day, Skin/gut/liver GvHD grades, gvhd_day,
gvhd_steroid_resistant, Mucositis_grade, BSI, Outcome_at_100).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Merging/data_dictionaries.xlsx
+++ b/Merging/data_dictionaries.xlsx
@@ -1717,6 +1717,11 @@
           <t>462 | 457 | 458 | 455 | 459</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Average read length (in base pairs) for the SRA run, computed as total bases / number of reads. Units: bp (integer).</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2076,6 +2081,16 @@
           <t>fastq,sra,run.zq | run.zq,sra,fastq | sra,fastq,run.zq | fastq,run.zq,sra | sra,run.zq,fastq</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>SRA internal metadata listing available download file formats for this run (e.g., fastq, sra, run.zq). Order within the string varies arbitrarily. Not analytically relevant.</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Redundant with DATASTORE provider and DATASTORE region — all three are SRA infrastructure columns with no analytical value. Could drop all three at harmonization.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2107,6 +2122,16 @@
           <t>ncbi,s3,gs | s3,gs,ncbi | s3,ncbi,gs | gs,s3,ncbi | ncbi,gs,s3</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>SRA internal metadata listing cloud storage providers hosting this run's files (ncbi = NCBI cold storage, s3 = AWS S3, gs = Google Cloud Storage). Not analytically relevant.</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Redundant with DATASTORE filetype and DATASTORE region — SRA infrastructure columns only.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2138,6 +2163,16 @@
           <t>s3.us-east-1,gs.us-east1,ncbi.public | ncbi.public,gs.us-east1,s3.us-east-1 | s3.us-east-1,ncbi.public,gs.us-east1 | gs.us-east1,ncbi.public,s3.us-east-1 | ncbi.public,s3.us-east-1,gs.us-east1</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>SRA internal metadata listing the specific cloud storage regions where this run's files are hosted (e.g., s3.us-east-1, gs.us-east1, ncbi.public). Not analytically relevant.</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Redundant with DATASTORE filetype and DATASTORE provider — SRA infrastructure columns only.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2825,6 +2860,11 @@
           <t>2019-12-03T00:00:00Z | 2019-12-05T00:00:00Z</t>
         </is>
       </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Date and time (ISO 8601 UTC) on which the SRA run record was made publicly available. Not analytically relevant; administrative SRA metadata.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2856,6 +2896,11 @@
           <t>2019-12-02T17:02:00Z | 2019-12-02T17:03:00Z</t>
         </is>
       </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Date and time (ISO 8601 UTC) on which the SRA run record was first created in the NCBI database. Not analytically relevant; administrative SRA metadata.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3051,6 +3096,16 @@
           <t>P5 | E1 | P4 | P3 | P2</t>
         </is>
       </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Study-assigned patient identifier. Prefix encodes nutritional group: E1–E10 = enteral nutrition (EN) group; P1–P10 = parenteral nutrition (PN) group. 20 unique patients, up to ~10 longitudinal samples each.</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Derived in Parsing_metadata.qmd by regex extraction from HostID (e.g., 'BP5PRE' → Patient 'P5').</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3082,6 +3137,16 @@
           <t>74 | 60 | 57 | 52 | 47</t>
         </is>
       </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Raw second run of digits extracted from the SRA HostID string by regex in Parsing_metadata.qmd (e.g., HostID 'BP5P74' → digits ['5','74'] → second_num = 74). For post-HSCT samples this equals the day post-HSCT embedded in the sample name. For pre-HSCT samples whose HostID contains 'PRE' (only one digit run), second_num is NA.</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>UNCERTAIN: the column is opaque and has no direct documentation. Basis: Parsing_metadata.qmd code `sapply(str_extract_all(HostID, '\\d+'), function(x) as.numeric(x[2]))`. Checked: manuscript, raw metadata headers — no explicit definition found. For post-HSCT rows, second_num == Timepoint; for pre-HSCT rows, second_num is NA and Timepoint uses the estimated_pre_day lookup. Recommend keeping Timepoint and dropping second_num at harmonization — it is purely an intermediate parsing artifact.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3113,6 +3178,16 @@
           <t>74 | 60 | 57 | 52 | 47</t>
         </is>
       </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Days relative to HSCT (day 0 = transplant day) for the fecal sample. Negative values are pre-HSCT sampling days (estimated from a patient-specific lookup table in Parsing_metadata.qmd, since SRA HostIDs for pre-HSCT samples only say 'PRE'). Positive values are post-HSCT days read directly from the HostID field. Units: days from HSCT; time origin = day of transplant (day 0). Range: approximately −18 to +120.</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Pre-HSCT day estimates are approximate — assigned from a handcoded lookup (pre_hsct_estimates in Parsing_metadata.qmd) rather than exact collection dates. For post-HSCT samples, Timepoint == second_num. The manuscript groups samples as: pre (&lt;0), HSCT (8–30 d), post40 (31–40 d), post60 (41–60 d), post120 (61–120 d).</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3144,6 +3219,16 @@
           <t>PN (+1/+36) | EN (+0/+18) | PN (+0/+18) | PN (+0/+16) | PN (+6/+19)</t>
         </is>
       </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Nutritional support regimen assigned to the patient immediately after HSCT. Format: 'type (+start/+end)', where type is EN (enteral nutrition / tube feeding) or PN (parenteral nutrition / intravenous), and +start/+end are days post-HSCT bounding the regimen. Patients with a single change have two segments separated by a semicolon. This is the primary between-group variable of the study: EN group (E1–E10) vs. PN group (P1–P10).</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Criterion for EN assignment: EN for ≥7 days post-HSCT. Criterion for PN assignment: total PN or EN &lt;7 days post-transplant (manuscript p.3).</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3175,6 +3260,11 @@
           <t>M | F</t>
         </is>
       </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Patient biological sex. M = male; F = female.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3206,6 +3296,11 @@
           <t>4 | 8 | 10 | 18 | 7</t>
         </is>
       </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Patient age at time of HSCT. Units: years (integer). Range: 1–18 years (all pediatric patients). Mean age: EN group 9.3 years, PN group 10.1 years (per manuscript).</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3237,6 +3332,16 @@
           <t>JMML | ALL B | AML | CGD | RCC</t>
         </is>
       </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Underlying hematologic or genetic disease for which the patient received HSCT. Values: ALL B = B-cell acute lymphoblastic leukemia; ALL T = T-cell acute lymphoblastic leukemia; AML = acute myeloid leukemia; CGD = chronic granulomatous disease; HLH = hemophagocytic lymphohistiocytosis; JMML = juvenile myelomonocytic leukemia; MDS = myelodysplastic syndrome; TM = thalassemia major; RCC = see notes.</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>UNCERTAIN: RCC expansion is ambiguous. In pediatric HSCT context, RCC most likely means 'refractory cytopenia of childhood' (a pediatric MDS subtype; per 2016 WHO classification), not 'renal cell carcinoma.' Basis: all other diagnoses are hematologic/genetic diseases amenable to HSCT in children; renal cell carcinoma would be atypical. Checked: manuscript text and abstract list the cohort as 'hematologic malignancies and hematological and genetic diseases'; Supplementary Table S2 (not available) would confirm. Recommend verifying against Supplementary Table S2 before finalizing.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3268,6 +3373,16 @@
           <t>MUD | Haploidentical | MFD | MMUD | MMFD</t>
         </is>
       </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Type of stem cell donor. MFD = matched family donor (HLA-matched related donor); MUD = matched unrelated donor; MMFD = mismatched family donor; MMUD = mismatched unrelated donor; Haploidentical = haploidentical donor (≥1 HLA antigen mismatch, typically a parent).</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>UNCERTAIN: MFD vs. MRD terminology varies; 'matched family donor' assumed equivalent to matched related donor (MRD) here. Basis: standard HSCT abbreviations; manuscript does not define abbreviations explicitly. Supplementary Table S2 would confirm.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3299,6 +3414,11 @@
           <t>BM | PBSC</t>
         </is>
       </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Source tissue from which hematopoietic stem cells were collected for transplantation. BM = bone marrow; PBSC = peripheral blood stem cells (mobilized by G-CSF).</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3330,6 +3450,16 @@
           <t>BU, EDX, L-PAM | BU, TT, FLUDARA | TREO, TT, FLUDARA | TREO, TT, EDX | BU, TT, EDX</t>
         </is>
       </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Pre-transplant myeloablative or reduced-intensity conditioning chemotherapy regimen, given as a comma-separated list of drug abbreviations. Drugs: BU = busulfan; TT = thiotepa; FLUDARA = fludarabine; EDX = cyclophosphamide (endoxan); L-PAM = melphalan; TREO = treosulfan; TBI = total body irradiation. Six distinct regimens observed.</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>UNCERTAIN: Drug abbreviation expansions are standard clinical/pharmacological abbreviations not defined in the manuscript. Basis: HSCT pharmacology conventions. TBI (total body irradiation) appears in one regimen ('EDX, FLUDARA, TBI') and is a radiation modality rather than a drug. Verified: manuscript mentions 'conditioning regimen' as a matching variable but does not list abbreviation definitions.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3361,6 +3491,16 @@
           <t>29 | 14 | 11 | 12 | 15</t>
         </is>
       </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Day post-HSCT on which neutrophil (PMN = polymorphonuclear) engraftment was achieved. Time origin = HSCT day 0; event = sustained neutrophil engraftment. Threshold: ANC ≥ 500 cells/μL (standard pediatric HSCT engraftment criterion). Units: days from HSCT (day 0). Range: 11–29 days.</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>UNCERTAIN: The exact engraftment threshold (ANC ≥ 500/μL) is the standard pediatric HSCT definition but is not stated explicitly in the manuscript. Checked: manuscript text and methods — engraftment criteria not defined. Supplementary Table S2 lists clinical data but is not available.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3392,6 +3532,16 @@
           <t>37 | 87 | 7 | 16 | 28</t>
         </is>
       </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Day post-HSCT on which platelet engraftment was achieved, defined as platelet count ≥ 20,000/μL without transfusion support. Time origin = HSCT day 0; event = platelet count ≥ 20,000/μL unsupported by transfusion. Units: days from HSCT (day 0). NA = not achieved within follow-up or censored (4 patients, 3.8% missing). Range: 7–87 days.</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Threshold is encoded in the column name (20,000/μL). The unsupported-by-transfusion criterion is standard but not explicitly stated in the manuscript. Column is patient-level (same value repeated across all samples from the same patient).</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3423,6 +3573,16 @@
           <t>0 | 2 | 3 | 1</t>
         </is>
       </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Maximum skin organ stage of acute GvHD (aGvHD) during follow-up, scored by the Glucksberg staging system. Scale: 0 = no skin involvement; 1 = Stage I (maculopapular rash &lt;25% BSA); 2 = Stage II (25–50% BSA); 3 = Stage III (&gt;50% BSA or generalized erythroderma). Patients without aGvHD scored 0.</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>UNCERTAIN: Glucksberg skin staging assumed; manuscript does not specify the grading system. The overall aGvHD grade (0–IV) is derived from the three organ stages (skin, gut, liver) but the overall grade column is not present — see gut_gvhd_grade and liver_gvhd_grade. These three organ-stage columns together constitute the Glucksberg organ staging input for computing overall aGvHD grade. Checked: manuscript mentions 'different grades of severity' and Supplementary Table S2 for clinical details; grading system not named in main text.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3454,6 +3614,16 @@
           <t>4 | 2 | 0 | 1 | 3</t>
         </is>
       </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Maximum gut organ stage of acute GvHD (aGvHD) during follow-up, scored by the Glucksberg staging system. Scale: 0 = no gut involvement; 1 = Stage I (diarrhea &gt;500 mL/day); 2 = Stage II (diarrhea &gt;1000 mL/day); 3 = Stage III (diarrhea &gt;1500 mL/day); 4 = Stage IV (severe abdominal pain ± ileus). Patients without aGvHD scored 0.</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>UNCERTAIN: Glucksberg gut staging assumed; see notes for Skin_gvhd_grade. One of three organ-stage columns (with Skin_gvhd_grade and liver_gvhd_grade) that together constitute the Glucksberg staging input. No overall GvHD grade column is present in this dataset.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3485,6 +3655,16 @@
           <t>0 | 3 | 2 | 1</t>
         </is>
       </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Maximum liver organ stage of acute GvHD (aGvHD) during follow-up, scored by the Glucksberg staging system. Scale: 0 = no liver involvement; 1 = Stage I (bilirubin 2–3 mg/dL); 2 = Stage II (bilirubin 3–6 mg/dL); 3 = Stage III (bilirubin 6–15 mg/dL). Patients without aGvHD scored 0. (Stage IV = bilirubin &gt;15 mg/dL, not observed.)</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>UNCERTAIN: Glucksberg liver staging assumed; see notes for Skin_gvhd_grade. One of three organ-stage columns (with Skin_gvhd_grade and gut_gvhd_grade) that together constitute the Glucksberg staging input. Overall GvHD grade not present as a separate column.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3516,6 +3696,16 @@
           <t>29 | 24 | 28 | 15 | 18</t>
         </is>
       </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Day post-HSCT on which acute GvHD was first clinically diagnosed. Time origin = HSCT day 0; event = first aGvHD diagnosis. Units: days from HSCT (day 0). Range among affected patients: 14–60 days. NA for patients who did not develop aGvHD (n ≈ 10 patients; 43.3% of samples missing).</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Missingness pattern mirrors gvhd_steroid_resistant: both are NA for GvHD-free patients (5/10 in each nutritional group per manuscript). The 43.3% missing at the sample level reflects repeated samples from the 10 non-GvHD patients.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3547,6 +3737,11 @@
           <t>y | n</t>
         </is>
       </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Whether the patient's acute GvHD was steroid-resistant (i.e., failed to respond to first-line corticosteroid therapy). y = steroid-resistant; n = steroid-responsive. NA for patients who did not develop aGvHD (same patients as gvhd_day = NA, 43.3% of samples).</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3578,6 +3773,16 @@
           <t>I | III | II | /</t>
         </is>
       </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Maximum grade of oral mucositis during the peri-transplant period, graded by WHO mucositis scale. Values: / = not graded or not recorded; I = Grade I (soreness ± erythema, able to eat); II = Grade II (erythema, ulcers, able to eat solids); III = Grade III (ulcers, requires liquid diet only). NA for 5 samples (4.8%).</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>UNCERTAIN: '/' value is ambiguous — may indicate Grade 0 (no mucositis) or missing/not recorded. Basis: WHO mucositis grading is standard for HSCT studies; value '/' does not map to any standard grade. Checked: manuscript mentions mucositis as a side effect of HSCT conditioning (p.2) but does not define the grading system or the '/' symbol. WHO scale also includes Grade IV (alimentation not possible) and Grade V (death); neither appears in data.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3609,6 +3814,16 @@
           <t>E.faecalis (+57); S.mitis (+57); S.orali | S.epidermidis (+6); E.faecalis (+6) | S.aureus (+7) | S.epidermidis (+5) | S.aureus (+94)</t>
         </is>
       </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Bloodstream infection(s) (BSI) documented during the transplant and follow-up period. Reported as organism name(s) followed by (+day), indicating the day post-HSCT of each BSI event. Multiple events separated by semicolons. NA = no BSI documented. Per manuscript, all 10 EN patients had no BSI; 7 of 10 PN patients had ≥1 BSI (11 total events). Organisms include Staphylococcus aureus, S. epidermidis, E. faecalis, S. mitis, S. oralis, K. pneumoniae, P. aeruginosa.</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>NA here means no BSI (not missing data) — confirmed by manuscript stating EN patients had 'no evidence of bloodstream infection.' BSI events in PN patients occurred mainly days +5 to +30 post-HSCT.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3638,6 +3853,11 @@
       <c r="G57" t="inlineStr">
         <is>
           <t>a | d</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Patient survival status at day +100 post-HSCT. a = alive at day +100; d = died before or at day +100. All 20 patients have a recorded value (no missing).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[Ingham] data dictionary meanings
</commit_message>
<xml_diff>
--- a/Merging/data_dictionaries.xlsx
+++ b/Merging/data_dictionaries.xlsx
@@ -5274,6 +5274,11 @@
           <t>P01 | P02 | P03 | P04 | P05</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Study-specific patient identifier (P01–P30); one patient may contribute multiple samples across timepoints.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5305,6 +5310,11 @@
           <t>8 | 16 | 21 | 36 | -6</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Days from transplant to stool sample collection (day 0 = transplant date). Integer; negative = pre-transplant. Renamed from days_posttransplant.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5336,6 +5346,11 @@
           <t>13-07-2010 | 21-07-2010 | 26-07-2010 | 10-08-2010 | 18-08-2010</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Calendar date of stool sample collection (dd-mm-yyyy).</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5367,6 +5382,11 @@
           <t>05-07-2010 | 24-08-2010 | 13-09-2010 | 15-09-2010 | 19-10-2010</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Calendar date of allogeneic stem cell transplant/BMT (dd-mm-yyyy). This is the time origin (day 0) for the timepoint column. Renamed from Date.of.BMT..dd.mm.yyyy.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5398,6 +5418,16 @@
           <t>1 | 2</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Transplant number for this patient: 1 = first allogeneic transplant, 2 = second allogeneic transplant.</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>UNCERTAIN: inferred from values (1 and 2 only) and standard EBMT registry field meaning. Checked manuscript and raw file headers; no explicit legend found.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5429,6 +5459,16 @@
           <t>14 | 300 | 402 | 24 | 571</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Numeric IBMTR disease code corresponding to the primary diagnosis. Text labels are in the disease column.</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Redundant with disease (numeric code vs text label). Prefer disease for harmonisation. UNCERTAIN: full IBMTR code table not reproduced in manuscript; codes inferred from paired disease text (e.g. DX=10 → AML, DX=24 → cALL, DX=300 → aplastic anaemia).</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5460,6 +5500,16 @@
           <t>AMML, M4 myelomonocytic | Severe aplastic anemia | Absence of T and B cells (SCID) | cALL (pre-B) | Fam. erythrophagocytic lymphohistiocytos</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Full IBMTR disease name for the primary diagnosis (free text from registry). E.g. 'cALL (pre-B)', 'Severe aplastic anemia', 'AML or ANLL, not otherwise specified'.</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Redundant with DX (text version). Prefer this column over DX for harmonisation because the text is self-documenting. Renamed from DiseaseNameIBMTR.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5491,6 +5541,11 @@
           <t>18-01-2010 | 08-06-2010 | 15-11-2009 | 15-11-2001 | 10-09-2010</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Calendar date of initial diagnosis (dd-mm-yyyy). Renamed from Date.of.diagnosis..dd.mm.yyyy.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5522,6 +5577,16 @@
           <t>2 | 1</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Donor sex (integer coded). By analogy with Sex (1=male, 2=female used in Parsing_metadata.qmd): 1 = male, 2 = female.</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>UNCERTAIN: coding 1=male/2=female is inferred from the Sex recoding in Parsing_metadata.qmd (case_when(Sex==1~'male', Sex==2~'female')). Donor.sex is not independently recoded in the script; checked manuscript — no explicit coding legend for Donor.sex.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5553,6 +5618,11 @@
           <t>7.490759754 | 14.6036961 | 1.196440794 | 11.57289528 | 1.188227242</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Recipient (patient) age at transplant in decimal years. Renamed from Rec.age.in.y.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5584,6 +5654,16 @@
           <t>20 | 89 | 7 | 31 | 9</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Patient body weight in kg (integer values). Reference point is pre-transplant (at time of conditioning).</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>UNCERTAIN: timepoint of weight measurement (pre-conditioning vs. transplant day) not stated explicitly in the manuscript. Inferred as pre-transplant from registry context.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5615,6 +5695,11 @@
           <t>30 | 42 | 37 | 41.90000153 | 20</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Donor age at time of donation in decimal years.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5646,6 +5731,16 @@
           <t>0 | 1</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>One-hot indicator: 1 = graft source is bone marrow (BM), 0 = not BM. Part of a one-hot graft-source group.</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>One-hot group: Bone.marrow / Peripheral.blood / Ubilical.cord (note: misspelled 'Ubilical' in original) encode a single underlying variable transplant_type. One patient (ERR2666891, P12) has both Bone.marrow=1 and Ubilical.cord=1, coded as BM_UC in transplant_type. Keep transplant_type for harmonisation; these three columns are the raw source.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5677,6 +5772,16 @@
           <t>0 | 1</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>One-hot indicator: 1 = graft source is peripheral blood stem cells (PBSC), 0 = not PBSC. Part of a one-hot graft-source group.</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>One-hot group: see Bone.marrow notes. Underlying variable: transplant_type.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5708,6 +5813,16 @@
           <t>1 | 0</t>
         </is>
       </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>One-hot indicator: 1 = graft source is umbilical cord blood (UC), 0 = not UC. Part of a one-hot graft-source group. Column name misspells 'umbilical' as 'ubilical' — preserved from original data.</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>One-hot group: see Bone.marrow notes. Underlying variable: transplant_type.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -5739,6 +5854,11 @@
           <t>2HLA_mismatch | matched_unrelated | sibling_donor | 1HLA_mismatch</t>
         </is>
       </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Donor–recipient HLA match classification. Values: matched_unrelated = fully HLA-matched unrelated donor; sibling_donor = HLA-identical sibling; 1HLA_mismatch = 1 antigen/allele mismatch; 2HLA_mismatch = 2 antigen/allele mismatches. Renamed from DonorMatch.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5770,6 +5890,11 @@
           <t>unrelated | sibling</t>
         </is>
       </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Donor type. Values: unrelated = volunteer unrelated donor; sibling = related sibling donor. Renamed from Donor.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5878,6 +6003,16 @@
           <t>2 | 1 | 3</t>
         </is>
       </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>CMV (cytomegalovirus) serostatus of donor–recipient pair. Values appear to be 1, 2, 3.</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>UNCERTAIN: exact coding not defined in manuscript or raw file headers. Common EBMT coding: 1 = R−/D− or D+/R−, 2 = R+ (recipient seropositive), 3 = mixed or indeterminate; however three-level coding may differ. Checked Data_matrix_37_patients.txt and Data_matrix_30_patients_additional.txt headers — no legend. Needs EBMT ProMISe codebook lookup.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5909,6 +6044,11 @@
           <t>1 | 0</t>
         </is>
       </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Binary indicator: acute GVHD occurred. 0 = no aGVHD, 1 = aGVHD occurred. Derived from EBMT field X541GVHDoccur.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -5940,6 +6080,11 @@
           <t>1 | 0 | 2 | 3 | 4</t>
         </is>
       </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Maximum acute GVHD grade (Glucksberg scale 0–IV). 0 = no aGVHD; 1 = grade I; 2 = grade II; 3 = grade III; 4 = grade IV. Derived from EBMT field X542MaxAGVHD.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -5971,6 +6116,11 @@
           <t>20-08-2010 | 06-10-2010 | 23-01-2011 | 05-02-2011 | 17-03-2011</t>
         </is>
       </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Calendar date of acute GVHD onset (dd-mm-yyyy). Missing for patients without aGVHD. Derived from EBMT field X549Date.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -6043,6 +6193,16 @@
           <t>22 | 70 | 10 | 900</t>
         </is>
       </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Coded primary cause of death. Values observed: 10, 22, 70, 900. Derived from Primary.cause.of.death.</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>UNCERTAIN: coding legend not reproduced in manuscript. Values look like EBMT ProMISe cause-of-death codes (e.g. 70 may = GVHD, 10 = relapse/progression, 22 = infection, 900 = other/unknown). Checked raw file headers — no legend. Needs EBMT ProMISe codebook lookup.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -6074,6 +6234,11 @@
           <t>2285.69669 | 9 | 2215.69669 | 2213.69669 | 2179.69669</t>
         </is>
       </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Time from transplant (day 0) to death or last follow-up (days). Event = death (see death column). Censored observations have tte_death equal to administrative follow-up time. Derived from EBMT field X.Alle..Survival.all.patients..to.death._Surv.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -6105,6 +6270,16 @@
           <t>1 | 0</t>
         </is>
       </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Overall survival censoring indicator (complement of death). 1 = alive/censored at tte_death; 0 = died. Equivalent to the original Alive...1.yes..0.no. column that was dropped during parsing.</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Redundant with death (Sens.death.0. = 1 − death). The Parsing_metadata.qmd script intended to drop it (the -Sens.death.0. inside the select(-c(...)) call is a double-negative that accidentally preserved the column). Prefer death for harmonisation. UNCERTAIN: the double-negative in select() is ambiguous — confirm intended behaviour.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -6136,6 +6311,11 @@
           <t>2285.69669 | 9 | 2215.69669 | 2213.69669 | 2179.69669</t>
         </is>
       </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Time from transplant (day 0) to treatment-related death (death in remission) or competing-event censoring (days). Event = tx_death. Competing events (relapse) are censored at the time of the competing event. Derived from EBMT field X.Alle..Death.in.remiss_Surv.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -6167,6 +6347,11 @@
           <t>2285.69669 | 9 | 2215.69669 | 2213.69669 | 2179.69669</t>
         </is>
       </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Time from transplant (day 0) to relapse or competing-event censoring (days). Event = relapse. Competing events (treatment-related death) are censored at the time of the competing event. Derived from EBMT field X.Alle..Relapse_Surv.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -6198,6 +6383,16 @@
           <t>2285.69669 | 2235.69669 | 2215.69669 | 2213.69669 | 2179.69669</t>
         </is>
       </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Administrative censoring time: days from transplant to database closure or end of observation window (Surv.to.now). This is the maximum observable follow-up time for each patient, irrespective of event status. Renamed from Surv.to.now.</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Not the time-to-event for any specific outcome — it is the ceiling follow-up time applied across all endpoints. For alive patients, tte_death = censor.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -6229,6 +6424,16 @@
           <t>0.63 | 5.857142857 | 3.870967742 | 5.333333333 | 1.281690141</t>
         </is>
       </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Infused cell dose per kg recipient body weight (×10^6/kg). Unit of cells not specified in the source file.</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>UNCERTAIN: numerator cell type (total mononuclear cells, CD34+ cells, or nucleated cells) not stated in raw data headers or manuscript methods. Checked Data_matrix_37_patients.txt and Data_matrix_30_patients_additional.txt — column name is Cell.dose.kg with no further annotation.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -6342,6 +6547,11 @@
           <t>0 | 1</t>
         </is>
       </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Binary indicator: irradiation was included in the conditioning regimen. 0 = no irradiation, 1 = irradiation given (includes TBI and/or other targeted irradiation).</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -6373,6 +6583,11 @@
           <t>0 | 1</t>
         </is>
       </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Binary indicator: total body irradiation (TBI) specifically was used in conditioning. 0 = no TBI, 1 = TBI given. Subset of Irrad.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -6404,6 +6619,11 @@
           <t>1200 | 200</t>
         </is>
       </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Total TBI dose in centigray (cGy). Missing for patients who did not receive TBI.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -6435,6 +6655,11 @@
           <t>1 | 0</t>
         </is>
       </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Binary indicator: TBI was delivered as fractionated (split) doses. 1 = fractionated TBI; 0 = single-dose (hyperfractionated or single-fraction) TBI.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -6466,6 +6691,11 @@
           <t>400 | 200</t>
         </is>
       </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Dose per TBI fraction in centigray (cGy). Missing for patients who did not receive fractionated TBI.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -6497,6 +6727,16 @@
           <t>1 | 0</t>
         </is>
       </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Binary indicator: anti-thymocyte globulin (ATG) was included in the conditioning regimen. 0 = no ATG, 1 = ATG given. Original column name in Data_matrix_37_patients.txt: ATGmm; prefixed X197 from EBMT ProMISe field numbering in the additional export.</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>UNCERTAIN: the 'mm' suffix in ATGmm is unexplained — may denote route, formulation (e.g. Micromet), or be an artefact of the EBMT field code. Exact EBMT field 197 definition not confirmed; inferred from paired column Total.dose.Busulfan..mg. context and binary values. Needs EBMT ProMISe codebook lookup.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -6528,6 +6768,16 @@
           <t>1 | 0 | 2</t>
         </is>
       </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Busulfan (Bu) use in conditioning. Original column: Bu in Data_matrix_37_patients.txt; EBMT field 233 in the additional export. Values: 0 = no busulfan; 1 = IV busulfan; 2 = oral busulfan (or alternative ordinal).</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>UNCERTAIN: coding 0/1/2 not defined in manuscript or raw headers. Three observed levels (0, 1, 2) suggest ordinal (route or dose tier) rather than binary. Needs EBMT ProMISe codebook lookup.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -6559,6 +6809,11 @@
           <t>350 | 144 | 179 | 193.92 | 365</t>
         </is>
       </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Total busulfan dose in mg administered as part of conditioning. Missing for patients not receiving busulfan.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -6590,6 +6845,11 @@
           <t>1 | 0</t>
         </is>
       </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Binary indicator: cyclophosphamide (Cyclo) included in conditioning. Original column: Cyclo in Data_matrix_37_patients.txt; EBMT field 270. 0 = no cyclophosphamide, 1 = cyclophosphamide given.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -6621,6 +6881,11 @@
           <t>2436 | 4600 | 2720 | 1800 | 8508</t>
         </is>
       </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Total cyclophosphamide dose in mg administered as part of conditioning. Missing for patients not receiving cyclophosphamide.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -6652,6 +6917,11 @@
           <t>1240 | 1480 | 373 | 1090 | 1600</t>
         </is>
       </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Total etoposide (VP-16) dose in mg administered as part of conditioning. Missing for patients not receiving etoposide.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -6683,6 +6953,11 @@
           <t>115 | 69 | 159 | 231 | 66</t>
         </is>
       </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Total melphalan dose in mg administered as part of conditioning. Missing for patients not receiving melphalan.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -6755,6 +7030,11 @@
           <t>0 | 1</t>
         </is>
       </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Binary indicator: fludarabine included in conditioning. Original column: Fludarab in Data_matrix_37_patients.txt; EBMT field 284.2. 0 = no fludarabine, 1 = fludarabine given.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -6786,6 +7066,16 @@
           <t>0 | 198 | 150 | 201 | 135</t>
         </is>
       </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Total fludarabine dose in mg as part of conditioning. Original column: TotalDoseFludarab in Data_matrix_37_patients.txt; EBMT field 284.3. Missing for patients not receiving fludarabine.</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>UNCERTAIN: unit (mg or mg/m²) not specified in raw headers. Inferred as mg from column name pattern matching Total.dose.Busulfan..mg. etc. Needs EBMT ProMISe codebook lookup.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -6817,6 +7107,16 @@
           <t>1 | 0</t>
         </is>
       </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Binary indicator: antibody-based conditioning agent included (e.g. Alemtuzumab/Campath or Rituximab). EBMT field 10; 'Ab' suffix = antibody. 0 = not given, 1 = given.</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>UNCERTAIN: specific antibody not identified. Not present in Data_matrix_37_patients.txt (only in the 30-patient additional EBMT export). Checked manuscript methods — no explicit mention of EBMT field 10. Needs EBMT ProMISe codebook lookup.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -6848,6 +7148,11 @@
           <t>50 | 90 | 80 | 100</t>
         </is>
       </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Karnofsky performance status score before start of conditioning. Scale 0–100 in 10-point increments; 100 = fully normal function, 0 = dead. Observed values: 50, 80, 90, 100.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -6879,6 +7184,11 @@
           <t>100 | 80 | 90</t>
         </is>
       </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Karnofsky performance status score at day 100 post-transplant. Scale 0–100. Missing for patients who died before day 100.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -6910,6 +7220,16 @@
           <t>1 | 0</t>
         </is>
       </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Binary indicator: successful engraftment achieved. 1 = engrafted, 0 = not engrafted. Column name preserves original spelling ('Engraphment' instead of 'Engraftment').</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>UNCERTAIN: engraftment definition (ANC &gt;0.5×10^9/L on 3 consecutive days, or other threshold) not stated in the manuscript. Checked raw file headers — no definition. Inferred binary meaning from values (0/1).</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -6941,6 +7261,16 @@
           <t>UC | PBSC | BM | BM_UC</t>
         </is>
       </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Graft source, derived in Parsing_metadata.qmd from Bone.marrow / Peripheral.blood / Ubilical.cord indicators. Values: BM = bone marrow; PBSC = peripheral blood stem cells; UC = umbilical cord blood; BM_UC = both BM and UC (one patient, ERR2666891).</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Derived column — see Bone.marrow, Peripheral.blood, Ubilical.cord for source. BM_UC is a special case hard-coded for ERR2666891.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -6972,6 +7302,11 @@
           <t>Cyclosporine + Corticosteroids | Cyclosporine A | Cyclosporine A + Methotrexate</t>
         </is>
       </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>GVHD prophylaxis regimen, decoded from GVHD.Prophylaxis integer in Parsing_metadata.qmd: 1 → 'Cyclosporine A'; 2 → 'Cyclosporine + Corticosteroids'; 7 → 'Cyclosporine A + Methotrexate'.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -7003,6 +7338,11 @@
           <t>female | male</t>
         </is>
       </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Recipient sex, decoded from Sex integer in Parsing_metadata.qmd: 1 → 'male'; 2 → 'female'.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -7034,6 +7374,11 @@
           <t>0 | 1</t>
         </is>
       </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Binary event indicator: patient died. Derived as 1 − Alive...1.yes..0.no. 0 = alive at last follow-up; 1 = died.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -7065,6 +7410,11 @@
           <t>0 | 1</t>
         </is>
       </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Binary event indicator: treatment-related death (death in remission). Derived as 1 − Sens.1.rel..now.0.death_remiss. 0 = no treatment-related death; 1 = died in remission.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -7094,6 +7444,11 @@
       <c r="G68" t="inlineStr">
         <is>
           <t>0 | 1</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Binary event indicator: disease relapse. Derived as 1 − Sens.0.relapse.1.death.Now. 0 = no relapse; 1 = relapsed.</t>
         </is>
       </c>
     </row>

</xml_diff>